<commit_message>
docs: record bounded P1 acceptance and Gate tracking (stage1)
</commit_message>
<xml_diff>
--- a/audit/canonical-candidate-20261019/proposed/FDS_P1_WBS_Status_Candidate_20261019.xlsx
+++ b/audit/canonical-candidate-20261019/proposed/FDS_P1_WBS_Status_Candidate_20261019.xlsx
@@ -2,16 +2,16 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Executive Summary" sheetId="1" r:id="R4a7e91e0e4d14e9d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="WBS" sheetId="2" r:id="Rd9aa271479dc4c51"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase 1 Gantt" sheetId="3" r:id="R26d74f51abaf449e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase 2 Gantt" sheetId="4" r:id="R88e4dac23fa14b62"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Milestones &amp; Decisions" sheetId="5" r:id="R79d3bd8f1a0844b5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risks &amp; Assumptions" sheetId="6" r:id="Rafa31320d2404be2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources &amp; Change Log" sheetId="7" r:id="R47ad5dcc595442ae"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Team Calendar" sheetId="8" r:id="R5fb07c33f51544f4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fast Track Plan" sheetId="9" r:id="Rc1cde953e3e747fa"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Strategy" sheetId="10" r:id="R3376edab031b4f98"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Executive Summary" sheetId="1" r:id="R63755d7f68304cbf"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="WBS" sheetId="2" r:id="R09423a91177b4ef2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase 1 Gantt" sheetId="3" r:id="Reaf68fc4e7074a0e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase 2 Gantt" sheetId="4" r:id="Rf604d847eae3403c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Milestones &amp; Decisions" sheetId="5" r:id="R15c6c0a69b244523"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risks &amp; Assumptions" sheetId="6" r:id="R8db3f7f8fab341e9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources &amp; Change Log" sheetId="7" r:id="R7baf2d391f5f413a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Team Calendar" sheetId="8" r:id="Rd09e61afcc5c47ff"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fast Track Plan" sheetId="9" r:id="Red818b1f18b74316"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Strategy" sheetId="10" r:id="R5cc9748f9af540f2"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1762,7 +1762,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rba381e022574406c"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R13271efd7e1f40b5"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1792,7 +1792,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rcb63c149bd574bf2"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R6ae52d8e18994510"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -2076,7 +2076,7 @@
     </x:row>
     <x:row r="2">
       <x:c r="A2" t="str">
-        <x:v>10/19 종결 7건만 반영. 다른 기록·계획은 10/03 기준 이력이며 전체 현행 WBS/새 정본이 아닙니다.</x:v>
+        <x:v>10/19 P1 선택11건 인수/상태 반영. 나머지67건·통제 표시는10/03 이력. P2입력은 별도. 전체 현행 WBS/새 정본 아님.</x:v>
       </x:c>
     </x:row>
     <x:row r="3">
@@ -2248,7 +2248,7 @@
       </x:c>
       <x:c r="B13" s="13" t="n">
         <x:f>COUNTIF(WBS!$G$4:$G$81,A13)</x:f>
-        <x:v>6</x:v>
+        <x:v>9</x:v>
       </x:c>
       <x:c r="D13" s="13" t="inlineStr">
         <x:is>
@@ -2288,7 +2288,7 @@
       </x:c>
       <x:c r="B15" s="13" t="n">
         <x:f>COUNTIF(WBS!$G$4:$G$81,A15)</x:f>
-        <x:v>37</x:v>
+        <x:v>34</x:v>
       </x:c>
     </x:row>
     <x:row r="16">
@@ -2495,7 +2495,7 @@
     <x:mergeCell ref="A18:V18"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R62f122c3516e453c"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R173b2fa03b204f62"/>
 </x:worksheet>
 </file>
 
@@ -3503,7 +3503,9 @@
         <x:v>Kubernetes 6개 Node의 보호 공백 없는 firewalld→Calico named HEP/GNP 전환, 30080/9100/10250 최소 허용, 관리망 반환 경로와 IF-06B 정합화, Positive/Negative/Regression/Reboot/Rollback 및 무결성 Evidence 완료</x:v>
       </x:c>
       <x:c r="Q11" s="195" t="str">
-        <x:v>09-21은 권장 Plan End이며 실제 종료일 확정이나 AC 완료가 아니다. 기존 End TBD 이력은 보존한다. CP→Worker·NTP·IF-16을 먼저, IF-06B·Negative/Reboot/Rollback·보호 인계를 후속 검증한다. 실제 상태·완료 판정은 유지한다. 세부 배정: Fast Track Plan 시트.
+        <x:v>10/19 조건부 인수/판정. 근거 https://github.com/321Team/fds-project-baseline/issues/14#issuecomment-6264595677. 현재 추적 반영 중, 티켓 OPEN. 원 AC/계획/Owner와 기술 한계 유지.
+[기존 계획/관측]
+09-21은 권장 Plan End이며 실제 종료일 확정이나 AC 완료가 아니다. 기존 End TBD 이력은 보존한다. CP→Worker·NTP·IF-16을 먼저, IF-06B·Negative/Reboot/Rollback·보호 인계를 후속 검증한다. 실제 상태·완료 판정은 유지한다. 세부 배정: Fast Track Plan 시트.
 GitHub open/-</x:v>
       </x:c>
       <x:c r="R11" s="13" t="str">
@@ -3792,7 +3794,7 @@
         <x:v>P0</x:v>
       </x:c>
       <x:c r="G16" s="13" t="str">
-        <x:v>To Do</x:v>
+        <x:v>In Progress</x:v>
       </x:c>
       <x:c r="H16" s="191" t="n">
         <x:v>46282</x:v>
@@ -3824,7 +3826,9 @@
         <x:v>CentOS/containerd, Ansible Inventory/SSH/멱등성, 3CP+3Worker, API LB/Calico, Harbor/Runner/PostgreSQL, Node Connectivity와 Push/Pull 준비도 승인</x:v>
       </x:c>
       <x:c r="Q16" s="195" t="str">
-        <x:v>09-17 오후 조건부 인수 목표. 6대·API/LB·Calico·DB·Harbor·Runner 증적 미충족이면 PASS 불가. 실제 상태·완료 판정은 유지한다. 세부 배정: Fast Track Plan 시트.
+        <x:v>10/19 조건부 인수/판정. 근거 https://github.com/321Team/fds-project-baseline/issues/18#issuecomment-6264597081. 현재 추적 반영 중, 티켓 OPEN. 원 AC/계획/Owner와 기술 한계 유지.
+[기존 계획/관측]
+09-17 오후 조건부 인수 목표. 6대·API/LB·Calico·DB·Harbor·Runner 증적 미충족이면 PASS 불가. 실제 상태·완료 판정은 유지한다. 세부 배정: Fast Track Plan 시트.
 GitHub open/-</x:v>
       </x:c>
       <x:c r="R16" s="13" t="str">
@@ -4112,7 +4116,7 @@
         <x:v>P0</x:v>
       </x:c>
       <x:c r="G21" s="13" t="str">
-        <x:v>To Do</x:v>
+        <x:v>In Progress</x:v>
       </x:c>
       <x:c r="H21" s="191" t="n">
         <x:v>46286</x:v>
@@ -4144,7 +4148,9 @@
         <x:v>2-Service MSA, DB 저장, Security P0, CI/CD, Monitoring, Initial E2E/Negative Test/Worker Drain 준비도를 승인</x:v>
       </x:c>
       <x:c r="Q21" s="195" t="str">
-        <x:v>09-21 오후 종료 시점 목표. 앱/보안/CI/Monitoring·초기 E2E/Negative/Drain 준비도와 해당 증적이 선행한다. 실제 상태·완료 판정은 유지한다. 세부 배정: Fast Track Plan 시트.
+        <x:v>10/19 조건부 인수/판정. 근거 https://github.com/321Team/fds-project-baseline/issues/23#issuecomment-6264221185. 현재 추적 반영 중, 티켓 OPEN. 원 AC/계획/Owner와 기술 한계 유지.
+[기존 계획/관측]
+09-21 오후 종료 시점 목표. 앱/보안/CI/Monitoring·초기 E2E/Negative/Drain 준비도와 해당 증적이 선행한다. 실제 상태·완료 판정은 유지한다. 세부 배정: Fast Track Plan 시트.
 GitHub open/-</x:v>
       </x:c>
       <x:c r="R21" s="13" t="str">
@@ -4477,7 +4483,7 @@
         <x:v>P0</x:v>
       </x:c>
       <x:c r="G27" s="13" t="str">
-        <x:v>To Do</x:v>
+        <x:v>In Progress</x:v>
       </x:c>
       <x:c r="H27" s="191" t="n">
         <x:v>46297</x:v>
@@ -4509,7 +4515,9 @@
         <x:v>Final E2E/Regression, Worker Drain, PostgreSQL Restore, Critical Issue 0, Architecture/Test/Runbook 준비도를 승인</x:v>
       </x:c>
       <x:c r="Q27" s="195" t="str">
-        <x:v>10-02는 실작업·증적 cutoff/G3 Review Ready 판정일이다. 남은 Phase 1 P0는 담당자별 공유 Runtime으로 직렬화하고, 미완료 AC는 10-06 Review에서 사실 상태를 분류한다. 일정 도래만으로 Gate PASS 처리하지 않는다.
+        <x:v>10/19 조건부 인수/판정. 근거 https://github.com/321Team/fds-project-baseline/issues/29#issuecomment-6264597709. 현재 추적 반영 중, 티켓 OPEN. 원 AC/계획/Owner와 기술 한계 유지.
+[기존 계획/관측]
+10-02는 실작업·증적 cutoff/G3 Review Ready 판정일이다. 남은 Phase 1 P0는 담당자별 공유 Runtime으로 직렬화하고, 미완료 AC는 10-06 Review에서 사실 상태를 분류한다. 일정 도래만으로 Gate PASS 처리하지 않는다.
 GitHub open/-</x:v>
       </x:c>
       <x:c r="R27" s="13" t="str">
@@ -7951,7 +7959,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7d7b5bf640a84d6e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R15ca3809d8374c98"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -9942,7 +9950,7 @@
       </x:c>
       <x:c r="C15" s="195" t="str">
         <x:f>WBS!G16</x:f>
-        <x:v>To Do</x:v>
+        <x:v>In Progress</x:v>
       </x:c>
       <x:c r="D15" s="225" t="n">
         <x:f>WBS!H16</x:f>
@@ -10780,7 +10788,7 @@
       </x:c>
       <x:c r="C20" s="195" t="str">
         <x:f>WBS!G21</x:f>
-        <x:v>To Do</x:v>
+        <x:v>In Progress</x:v>
       </x:c>
       <x:c r="D20" s="225" t="n">
         <x:f>WBS!H21</x:f>
@@ -11756,7 +11764,7 @@
       </x:c>
       <x:c r="C26" s="195" t="str">
         <x:f>WBS!G27</x:f>
-        <x:v>To Do</x:v>
+        <x:v>In Progress</x:v>
       </x:c>
       <x:c r="D26" s="225" t="n">
         <x:f>WBS!H27</x:f>
@@ -25483,7 +25491,7 @@
       </x:c>
       <x:c r="D6" s="13" t="str">
         <x:f>WBS!G16</x:f>
-        <x:v>To Do</x:v>
+        <x:v>In Progress</x:v>
       </x:c>
       <x:c r="E6" s="191" t="n">
         <x:f>WBS!H16</x:f>
@@ -25502,7 +25510,9 @@
       </x:c>
       <x:c r="I6" s="195" t="str">
         <x:f>WBS!Q16</x:f>
-        <x:v>09-17 오후 조건부 인수 목표. 6대·API/LB·Calico·DB·Harbor·Runner 증적 미충족이면 PASS 불가. 실제 상태·완료 판정은 유지한다. 세부 배정: Fast Track Plan 시트.
+        <x:v>10/19 조건부 인수/판정. 근거 https://github.com/321Team/fds-project-baseline/issues/18#issuecomment-6264597081. 현재 추적 반영 중, 티켓 OPEN. 원 AC/계획/Owner와 기술 한계 유지.
+[기존 계획/관측]
+09-17 오후 조건부 인수 목표. 6대·API/LB·Calico·DB·Harbor·Runner 증적 미충족이면 PASS 불가. 실제 상태·완료 판정은 유지한다. 세부 배정: Fast Track Plan 시트.
 GitHub open/-</x:v>
       </x:c>
       <x:c r="J6" s="195" t="str">
@@ -25524,7 +25534,7 @@
       </x:c>
       <x:c r="D7" s="13" t="str">
         <x:f>WBS!G21</x:f>
-        <x:v>To Do</x:v>
+        <x:v>In Progress</x:v>
       </x:c>
       <x:c r="E7" s="191" t="n">
         <x:f>WBS!H21</x:f>
@@ -25543,7 +25553,9 @@
       </x:c>
       <x:c r="I7" s="195" t="str">
         <x:f>WBS!Q21</x:f>
-        <x:v>09-21 오후 종료 시점 목표. 앱/보안/CI/Monitoring·초기 E2E/Negative/Drain 준비도와 해당 증적이 선행한다. 실제 상태·완료 판정은 유지한다. 세부 배정: Fast Track Plan 시트.
+        <x:v>10/19 조건부 인수/판정. 근거 https://github.com/321Team/fds-project-baseline/issues/23#issuecomment-6264221185. 현재 추적 반영 중, 티켓 OPEN. 원 AC/계획/Owner와 기술 한계 유지.
+[기존 계획/관측]
+09-21 오후 종료 시점 목표. 앱/보안/CI/Monitoring·초기 E2E/Negative/Drain 준비도와 해당 증적이 선행한다. 실제 상태·완료 판정은 유지한다. 세부 배정: Fast Track Plan 시트.
 GitHub open/-</x:v>
       </x:c>
       <x:c r="J7" s="195" t="str">
@@ -25606,7 +25618,7 @@
       </x:c>
       <x:c r="D9" s="13" t="str">
         <x:f>WBS!G27</x:f>
-        <x:v>To Do</x:v>
+        <x:v>In Progress</x:v>
       </x:c>
       <x:c r="E9" s="191" t="n">
         <x:f>WBS!H27</x:f>
@@ -25625,7 +25637,9 @@
       </x:c>
       <x:c r="I9" s="195" t="str">
         <x:f>WBS!Q27</x:f>
-        <x:v>10-02는 실작업·증적 cutoff/G3 Review Ready 판정일이다. 남은 Phase 1 P0는 담당자별 공유 Runtime으로 직렬화하고, 미완료 AC는 10-06 Review에서 사실 상태를 분류한다. 일정 도래만으로 Gate PASS 처리하지 않는다.
+        <x:v>10/19 조건부 인수/판정. 근거 https://github.com/321Team/fds-project-baseline/issues/29#issuecomment-6264597709. 현재 추적 반영 중, 티켓 OPEN. 원 AC/계획/Owner와 기술 한계 유지.
+[기존 계획/관측]
+10-02는 실작업·증적 cutoff/G3 Review Ready 판정일이다. 남은 Phase 1 P0는 담당자별 공유 Runtime으로 직렬화하고, 미완료 AC는 10-06 Review에서 사실 상태를 분류한다. 일정 도래만으로 Gate PASS 처리하지 않는다.
 GitHub open/-</x:v>
       </x:c>
       <x:c r="J9" s="195" t="str">

</xml_diff>

<commit_message>
docs: record bounded P1 acceptance and Gate tracking (stage2)
</commit_message>
<xml_diff>
--- a/audit/canonical-candidate-20261019/proposed/FDS_P1_WBS_Status_Candidate_20261019.xlsx
+++ b/audit/canonical-candidate-20261019/proposed/FDS_P1_WBS_Status_Candidate_20261019.xlsx
@@ -2,16 +2,16 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Executive Summary" sheetId="1" r:id="R63755d7f68304cbf"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="WBS" sheetId="2" r:id="R09423a91177b4ef2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase 1 Gantt" sheetId="3" r:id="Reaf68fc4e7074a0e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase 2 Gantt" sheetId="4" r:id="Rf604d847eae3403c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Milestones &amp; Decisions" sheetId="5" r:id="R15c6c0a69b244523"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risks &amp; Assumptions" sheetId="6" r:id="R8db3f7f8fab341e9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources &amp; Change Log" sheetId="7" r:id="R7baf2d391f5f413a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Team Calendar" sheetId="8" r:id="Rd09e61afcc5c47ff"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fast Track Plan" sheetId="9" r:id="Red818b1f18b74316"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Strategy" sheetId="10" r:id="R5cc9748f9af540f2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Executive Summary" sheetId="1" r:id="Rd47ecd3372aa4c70"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="WBS" sheetId="2" r:id="R26fec5354633485c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase 1 Gantt" sheetId="3" r:id="Re8c39cdf51ac47fc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase 2 Gantt" sheetId="4" r:id="R43a9ff5811a840c0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Milestones &amp; Decisions" sheetId="5" r:id="Rd1c92d395caf4252"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risks &amp; Assumptions" sheetId="6" r:id="R2020d8cf5d844c87"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources &amp; Change Log" sheetId="7" r:id="Rbaeb74642f3145ec"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Team Calendar" sheetId="8" r:id="R683b47f41ecf4811"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fast Track Plan" sheetId="9" r:id="Rc66a6fa8b21f4c40"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Strategy" sheetId="10" r:id="Re7d064832d6443bc"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1762,7 +1762,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R13271efd7e1f40b5"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Re7831b5302e2498d"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1792,7 +1792,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R6ae52d8e18994510"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rda20770f7890467b"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -2228,7 +2228,7 @@
       </x:c>
       <x:c r="B12" s="13" t="n">
         <x:f>COUNTIF(WBS!$G$4:$G$81,A12)</x:f>
-        <x:v>34</x:v>
+        <x:v>38</x:v>
       </x:c>
       <x:c r="D12" s="13" t="inlineStr">
         <x:is>
@@ -2248,7 +2248,7 @@
       </x:c>
       <x:c r="B13" s="13" t="n">
         <x:f>COUNTIF(WBS!$G$4:$G$81,A13)</x:f>
-        <x:v>9</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="D13" s="13" t="inlineStr">
         <x:is>
@@ -2495,7 +2495,7 @@
     <x:mergeCell ref="A18:V18"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R173b2fa03b204f62"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R56581ba0662c47bb"/>
 </x:worksheet>
 </file>
 
@@ -3471,7 +3471,7 @@
         <x:v>P0</x:v>
       </x:c>
       <x:c r="G11" s="13" t="str">
-        <x:v>In Progress</x:v>
+        <x:v>Done</x:v>
       </x:c>
       <x:c r="H11" s="191" t="n">
         <x:v>46266</x:v>
@@ -3503,7 +3503,7 @@
         <x:v>Kubernetes 6개 Node의 보호 공백 없는 firewalld→Calico named HEP/GNP 전환, 30080/9100/10250 최소 허용, 관리망 반환 경로와 IF-06B 정합화, Positive/Negative/Regression/Reboot/Rollback 및 무결성 Evidence 완료</x:v>
       </x:c>
       <x:c r="Q11" s="195" t="str">
-        <x:v>10/19 조건부 인수/판정. 근거 https://github.com/321Team/fds-project-baseline/issues/14#issuecomment-6264595677. 현재 추적 반영 중, 티켓 OPEN. 원 AC/계획/Owner와 기술 한계 유지.
+        <x:v>10/19 조건부 인수/판정. 근거 https://github.com/321Team/fds-project-baseline/issues/14#issuecomment-6264595677. 실제 종결 2026-10-19T19:05:24+09:00. 종결 근거 https://github.com/321Team/fds-project-baseline/issues/14#issuecomment-6264705121. 원 AC/계획/Owner와 기술 한계 유지.
 [기존 계획/관측]
 09-21은 권장 Plan End이며 실제 종료일 확정이나 AC 완료가 아니다. 기존 End TBD 이력은 보존한다. CP→Worker·NTP·IF-16을 먼저, IF-06B·Negative/Reboot/Rollback·보호 인계를 후속 검증한다. 실제 상태·완료 판정은 유지한다. 세부 배정: Fast Track Plan 시트.
 GitHub open/-</x:v>
@@ -3513,7 +3513,7 @@
       </x:c>
       <x:c r="S11" s="13" t="str">
         <x:f>IF(G11="Done","Done",IF(I11="","End TBD",IF(I11&lt;'Executive Summary'!$B$4,"Target elapsed",IF(H11&gt;'Executive Summary'!$B$4,"Upcoming","Active window"))))</x:f>
-        <x:v>Target elapsed</x:v>
+        <x:v>Done</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="110" customHeight="1">
@@ -3794,7 +3794,7 @@
         <x:v>P0</x:v>
       </x:c>
       <x:c r="G16" s="13" t="str">
-        <x:v>In Progress</x:v>
+        <x:v>Done</x:v>
       </x:c>
       <x:c r="H16" s="191" t="n">
         <x:v>46282</x:v>
@@ -3826,7 +3826,7 @@
         <x:v>CentOS/containerd, Ansible Inventory/SSH/멱등성, 3CP+3Worker, API LB/Calico, Harbor/Runner/PostgreSQL, Node Connectivity와 Push/Pull 준비도 승인</x:v>
       </x:c>
       <x:c r="Q16" s="195" t="str">
-        <x:v>10/19 조건부 인수/판정. 근거 https://github.com/321Team/fds-project-baseline/issues/18#issuecomment-6264597081. 현재 추적 반영 중, 티켓 OPEN. 원 AC/계획/Owner와 기술 한계 유지.
+        <x:v>10/19 조건부 인수/판정. 근거 https://github.com/321Team/fds-project-baseline/issues/18#issuecomment-6264597081. 실제 종결 2026-10-19T19:05:40+09:00. 종결 근거 https://github.com/321Team/fds-project-baseline/issues/18#issuecomment-6264709975. 원 AC/계획/Owner와 기술 한계 유지.
 [기존 계획/관측]
 09-17 오후 조건부 인수 목표. 6대·API/LB·Calico·DB·Harbor·Runner 증적 미충족이면 PASS 불가. 실제 상태·완료 판정은 유지한다. 세부 배정: Fast Track Plan 시트.
 GitHub open/-</x:v>
@@ -3836,7 +3836,7 @@
       </x:c>
       <x:c r="S16" s="13" t="str">
         <x:f>IF(G16="Done","Done",IF(I16="","End TBD",IF(I16&lt;'Executive Summary'!$B$4,"Target elapsed",IF(H16&gt;'Executive Summary'!$B$4,"Upcoming","Active window"))))</x:f>
-        <x:v>Target elapsed</x:v>
+        <x:v>Done</x:v>
       </x:c>
     </x:row>
     <x:row r="17" ht="110" customHeight="1">
@@ -4116,7 +4116,7 @@
         <x:v>P0</x:v>
       </x:c>
       <x:c r="G21" s="13" t="str">
-        <x:v>In Progress</x:v>
+        <x:v>Done</x:v>
       </x:c>
       <x:c r="H21" s="191" t="n">
         <x:v>46286</x:v>
@@ -4148,7 +4148,7 @@
         <x:v>2-Service MSA, DB 저장, Security P0, CI/CD, Monitoring, Initial E2E/Negative Test/Worker Drain 준비도를 승인</x:v>
       </x:c>
       <x:c r="Q21" s="195" t="str">
-        <x:v>10/19 조건부 인수/판정. 근거 https://github.com/321Team/fds-project-baseline/issues/23#issuecomment-6264221185. 현재 추적 반영 중, 티켓 OPEN. 원 AC/계획/Owner와 기술 한계 유지.
+        <x:v>10/19 조건부 인수/판정. 근거 https://github.com/321Team/fds-project-baseline/issues/23#issuecomment-6264221185. 실제 종결 2026-10-19T19:05:48+09:00. 종결 근거 https://github.com/321Team/fds-project-baseline/issues/23#issuecomment-6264712221. 원 AC/계획/Owner와 기술 한계 유지.
 [기존 계획/관측]
 09-21 오후 종료 시점 목표. 앱/보안/CI/Monitoring·초기 E2E/Negative/Drain 준비도와 해당 증적이 선행한다. 실제 상태·완료 판정은 유지한다. 세부 배정: Fast Track Plan 시트.
 GitHub open/-</x:v>
@@ -4158,7 +4158,7 @@
       </x:c>
       <x:c r="S21" s="13" t="str">
         <x:f>IF(G21="Done","Done",IF(I21="","End TBD",IF(I21&lt;'Executive Summary'!$B$4,"Target elapsed",IF(H21&gt;'Executive Summary'!$B$4,"Upcoming","Active window"))))</x:f>
-        <x:v>Target elapsed</x:v>
+        <x:v>Done</x:v>
       </x:c>
     </x:row>
     <x:row r="22" ht="110" customHeight="1">
@@ -4483,7 +4483,7 @@
         <x:v>P0</x:v>
       </x:c>
       <x:c r="G27" s="13" t="str">
-        <x:v>In Progress</x:v>
+        <x:v>Done</x:v>
       </x:c>
       <x:c r="H27" s="191" t="n">
         <x:v>46297</x:v>
@@ -4515,7 +4515,7 @@
         <x:v>Final E2E/Regression, Worker Drain, PostgreSQL Restore, Critical Issue 0, Architecture/Test/Runbook 준비도를 승인</x:v>
       </x:c>
       <x:c r="Q27" s="195" t="str">
-        <x:v>10/19 조건부 인수/판정. 근거 https://github.com/321Team/fds-project-baseline/issues/29#issuecomment-6264597709. 현재 추적 반영 중, 티켓 OPEN. 원 AC/계획/Owner와 기술 한계 유지.
+        <x:v>10/19 조건부 인수/판정. 근거 https://github.com/321Team/fds-project-baseline/issues/29#issuecomment-6264597709. 실제 종결 2026-10-19T19:05:55+09:00. 종결 근거 https://github.com/321Team/fds-project-baseline/issues/29#issuecomment-6264714186. 원 AC/계획/Owner와 기술 한계 유지.
 [기존 계획/관측]
 10-02는 실작업·증적 cutoff/G3 Review Ready 판정일이다. 남은 Phase 1 P0는 담당자별 공유 Runtime으로 직렬화하고, 미완료 AC는 10-06 Review에서 사실 상태를 분류한다. 일정 도래만으로 Gate PASS 처리하지 않는다.
 GitHub open/-</x:v>
@@ -4525,7 +4525,7 @@
       </x:c>
       <x:c r="S27" s="13" t="str">
         <x:f>IF(G27="Done","Done",IF(I27="","End TBD",IF(I27&lt;'Executive Summary'!$B$4,"Target elapsed",IF(H27&gt;'Executive Summary'!$B$4,"Upcoming","Active window"))))</x:f>
-        <x:v>Target elapsed</x:v>
+        <x:v>Done</x:v>
       </x:c>
     </x:row>
     <x:row r="28" ht="110" customHeight="1">
@@ -7959,7 +7959,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R15ca3809d8374c98"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5a212b11954840f6"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -9104,7 +9104,7 @@
       </x:c>
       <x:c r="C10" s="195" t="str">
         <x:f>WBS!G11</x:f>
-        <x:v>In Progress</x:v>
+        <x:v>Done</x:v>
       </x:c>
       <x:c r="D10" s="225" t="n">
         <x:f>WBS!H11</x:f>
@@ -9950,7 +9950,7 @@
       </x:c>
       <x:c r="C15" s="195" t="str">
         <x:f>WBS!G16</x:f>
-        <x:v>In Progress</x:v>
+        <x:v>Done</x:v>
       </x:c>
       <x:c r="D15" s="225" t="n">
         <x:f>WBS!H16</x:f>
@@ -10788,7 +10788,7 @@
       </x:c>
       <x:c r="C20" s="195" t="str">
         <x:f>WBS!G21</x:f>
-        <x:v>In Progress</x:v>
+        <x:v>Done</x:v>
       </x:c>
       <x:c r="D20" s="225" t="n">
         <x:f>WBS!H21</x:f>
@@ -11764,7 +11764,7 @@
       </x:c>
       <x:c r="C26" s="195" t="str">
         <x:f>WBS!G27</x:f>
-        <x:v>In Progress</x:v>
+        <x:v>Done</x:v>
       </x:c>
       <x:c r="D26" s="225" t="n">
         <x:f>WBS!H27</x:f>
@@ -25491,7 +25491,7 @@
       </x:c>
       <x:c r="D6" s="13" t="str">
         <x:f>WBS!G16</x:f>
-        <x:v>In Progress</x:v>
+        <x:v>Done</x:v>
       </x:c>
       <x:c r="E6" s="191" t="n">
         <x:f>WBS!H16</x:f>
@@ -25510,7 +25510,7 @@
       </x:c>
       <x:c r="I6" s="195" t="str">
         <x:f>WBS!Q16</x:f>
-        <x:v>10/19 조건부 인수/판정. 근거 https://github.com/321Team/fds-project-baseline/issues/18#issuecomment-6264597081. 현재 추적 반영 중, 티켓 OPEN. 원 AC/계획/Owner와 기술 한계 유지.
+        <x:v>10/19 조건부 인수/판정. 근거 https://github.com/321Team/fds-project-baseline/issues/18#issuecomment-6264597081. 실제 종결 2026-10-19T19:05:40+09:00. 종결 근거 https://github.com/321Team/fds-project-baseline/issues/18#issuecomment-6264709975. 원 AC/계획/Owner와 기술 한계 유지.
 [기존 계획/관측]
 09-17 오후 조건부 인수 목표. 6대·API/LB·Calico·DB·Harbor·Runner 증적 미충족이면 PASS 불가. 실제 상태·완료 판정은 유지한다. 세부 배정: Fast Track Plan 시트.
 GitHub open/-</x:v>
@@ -25534,7 +25534,7 @@
       </x:c>
       <x:c r="D7" s="13" t="str">
         <x:f>WBS!G21</x:f>
-        <x:v>In Progress</x:v>
+        <x:v>Done</x:v>
       </x:c>
       <x:c r="E7" s="191" t="n">
         <x:f>WBS!H21</x:f>
@@ -25553,7 +25553,7 @@
       </x:c>
       <x:c r="I7" s="195" t="str">
         <x:f>WBS!Q21</x:f>
-        <x:v>10/19 조건부 인수/판정. 근거 https://github.com/321Team/fds-project-baseline/issues/23#issuecomment-6264221185. 현재 추적 반영 중, 티켓 OPEN. 원 AC/계획/Owner와 기술 한계 유지.
+        <x:v>10/19 조건부 인수/판정. 근거 https://github.com/321Team/fds-project-baseline/issues/23#issuecomment-6264221185. 실제 종결 2026-10-19T19:05:48+09:00. 종결 근거 https://github.com/321Team/fds-project-baseline/issues/23#issuecomment-6264712221. 원 AC/계획/Owner와 기술 한계 유지.
 [기존 계획/관측]
 09-21 오후 종료 시점 목표. 앱/보안/CI/Monitoring·초기 E2E/Negative/Drain 준비도와 해당 증적이 선행한다. 실제 상태·완료 판정은 유지한다. 세부 배정: Fast Track Plan 시트.
 GitHub open/-</x:v>
@@ -25618,7 +25618,7 @@
       </x:c>
       <x:c r="D9" s="13" t="str">
         <x:f>WBS!G27</x:f>
-        <x:v>In Progress</x:v>
+        <x:v>Done</x:v>
       </x:c>
       <x:c r="E9" s="191" t="n">
         <x:f>WBS!H27</x:f>
@@ -25637,7 +25637,7 @@
       </x:c>
       <x:c r="I9" s="195" t="str">
         <x:f>WBS!Q27</x:f>
-        <x:v>10/19 조건부 인수/판정. 근거 https://github.com/321Team/fds-project-baseline/issues/29#issuecomment-6264597709. 현재 추적 반영 중, 티켓 OPEN. 원 AC/계획/Owner와 기술 한계 유지.
+        <x:v>10/19 조건부 인수/판정. 근거 https://github.com/321Team/fds-project-baseline/issues/29#issuecomment-6264597709. 실제 종결 2026-10-19T19:05:55+09:00. 종결 근거 https://github.com/321Team/fds-project-baseline/issues/29#issuecomment-6264714186. 원 AC/계획/Owner와 기술 한계 유지.
 [기존 계획/관측]
 10-02는 실작업·증적 cutoff/G3 Review Ready 판정일이다. 남은 Phase 1 P0는 담당자별 공유 Runtime으로 직렬화하고, 미완료 AC는 10-06 Review에서 사실 상태를 분류한다. 일정 도래만으로 Gate PASS 처리하지 않는다.
 GitHub open/-</x:v>

</xml_diff>

<commit_message>
docs: integrate all78 WBS and approved Phase2 specifications in candidate
</commit_message>
<xml_diff>
--- a/audit/canonical-candidate-20261019/proposed/FDS_P1_WBS_Status_Candidate_20261019.xlsx
+++ b/audit/canonical-candidate-20261019/proposed/FDS_P1_WBS_Status_Candidate_20261019.xlsx
@@ -2,16 +2,16 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Executive Summary" sheetId="1" r:id="Rd47ecd3372aa4c70"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="WBS" sheetId="2" r:id="R26fec5354633485c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase 1 Gantt" sheetId="3" r:id="Re8c39cdf51ac47fc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase 2 Gantt" sheetId="4" r:id="R43a9ff5811a840c0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Milestones &amp; Decisions" sheetId="5" r:id="Rd1c92d395caf4252"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risks &amp; Assumptions" sheetId="6" r:id="R2020d8cf5d844c87"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources &amp; Change Log" sheetId="7" r:id="Rbaeb74642f3145ec"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Team Calendar" sheetId="8" r:id="R683b47f41ecf4811"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fast Track Plan" sheetId="9" r:id="Rc66a6fa8b21f4c40"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Strategy" sheetId="10" r:id="Re7d064832d6443bc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Executive Summary" sheetId="1" r:id="R42f3e076264c4eb7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="WBS" sheetId="2" r:id="R708f3804f8e6408c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase 1 Gantt" sheetId="3" r:id="R4e0843d731ce47b5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase 2 Gantt" sheetId="4" r:id="Ra8c9a790392e4347"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Milestones &amp; Decisions" sheetId="5" r:id="Ra5a5e20e8aa84886"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risks &amp; Assumptions" sheetId="6" r:id="R90958ae79ffe4113"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources &amp; Change Log" sheetId="7" r:id="Rf58d195b06d04aba"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Team Calendar" sheetId="8" r:id="R0d32c6285c854eb5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fast Track Plan" sheetId="9" r:id="Ra558d84348154995"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Strategy" sheetId="10" r:id="R48c9a11a844e4559"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1762,7 +1762,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Re7831b5302e2498d"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R1124a92c80e944b1"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1792,7 +1792,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rda20770f7890467b"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Re4c0e19a97d644de"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -2050,7 +2050,7 @@
   <x:sheetData>
     <x:row r="1" ht="32" customHeight="1">
       <x:c r="A1" s="237" t="str">
-        <x:v>FDS v3.1.21 · Executive Summary 기반 후속 후보</x:v>
+        <x:v>FDS 전체 WBS · Phase1·2 정본 후보</x:v>
       </x:c>
       <x:c r="B1" s="238"/>
       <x:c r="C1" s="238"/>
@@ -2076,7 +2076,7 @@
     </x:row>
     <x:row r="2">
       <x:c r="A2" t="str">
-        <x:v>10/19 P1 선택11건 인수/상태 반영. 나머지67건·통제 표시는10/03 이력. P2입력은 별도. 전체 현행 WBS/새 정본 아님.</x:v>
+        <x:v>78건 현재 GitHub 상태 반영. Phase2 사양 확정과 Runtime 인수 구분. 계획일은 승인된 이력이며 실제 완료일은 R열. 미발행 후보.</x:v>
       </x:c>
     </x:row>
     <x:row r="3">
@@ -2107,14 +2107,14 @@
           <x:t xml:space="preserve">As of</x:t>
         </x:is>
       </x:c>
-      <x:c r="B4" s="154" t="n">
-        <x:v>46298</x:v>
+      <x:c r="B4" s="154" t="d">
+        <x:v>2026-10-19T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="D4" s="13" t="str">
         <x:v>P1 Close</x:v>
       </x:c>
       <x:c r="E4" s="199" t="str">
-        <x:v>HOLD · 10/6 review</x:v>
+        <x:v>Review 진행 · Signoff 미완료</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="32" customHeight="1">
@@ -2124,13 +2124,13 @@
         </x:is>
       </x:c>
       <x:c r="B5" s="195" t="str">
-        <x:v>v3.1.21 RELEASED</x:v>
+        <x:v>v3.1.21 기반 · 미발행 후보</x:v>
       </x:c>
       <x:c r="D5" s="13" t="str">
         <x:v>D21 decision</x:v>
       </x:c>
       <x:c r="E5" s="199" t="str">
-        <x:v>FINAL · 10/3</x:v>
+        <x:v>FINAL · AWS EC2 Relay</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
@@ -2147,7 +2147,7 @@
         <x:v>D21 publication</x:v>
       </x:c>
       <x:c r="E6" s="199" t="str">
-        <x:v>HOLD · raw intake</x:v>
+        <x:v>사양 후보 편입 · 새 Release 없음</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
@@ -2164,7 +2164,7 @@
         <x:v>Architecture Freeze</x:v>
       </x:c>
       <x:c r="E7" s="199" t="str">
-        <x:v>HOLD</x:v>
+        <x:v>P1 문서 한정 / P2 설계 Freeze</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
@@ -2181,21 +2181,21 @@
         <x:v>Stage-A</x:v>
       </x:c>
       <x:c r="E8" s="199" t="str">
-        <x:v>NOT_READY</x:v>
+        <x:v>당시 NOT_READY · 현재 GO 미판정</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
       <x:c r="A9" t="str">
-        <x:v>Rows / Milestone</x:v>
+        <x:v>Phase 1 / Phase 2</x:v>
       </x:c>
       <x:c r="B9" t="str">
-        <x:v>78 / 76</x:v>
+        <x:v>42 / 31</x:v>
       </x:c>
       <x:c r="D9" s="67" t="str">
         <x:v>G4 / G5 / G6 targets</x:v>
       </x:c>
       <x:c r="E9" s="200" t="str">
-        <x:v>10/14 · 10/20 · 10/22</x:v>
+        <x:v>원 계획 유지 · 실제 인수 별도</x:v>
       </x:c>
     </x:row>
     <x:row r="11">
@@ -2228,7 +2228,7 @@
       </x:c>
       <x:c r="B12" s="13" t="n">
         <x:f>COUNTIF(WBS!$G$4:$G$81,A12)</x:f>
-        <x:v>38</x:v>
+        <x:v>42</x:v>
       </x:c>
       <x:c r="D12" s="13" t="inlineStr">
         <x:is>
@@ -2248,7 +2248,7 @@
       </x:c>
       <x:c r="B13" s="13" t="n">
         <x:f>COUNTIF(WBS!$G$4:$G$81,A13)</x:f>
-        <x:v>5</x:v>
+        <x:v>13</x:v>
       </x:c>
       <x:c r="D13" s="13" t="inlineStr">
         <x:is>
@@ -2288,16 +2288,16 @@
       </x:c>
       <x:c r="B15" s="13" t="n">
         <x:f>COUNTIF(WBS!$G$4:$G$81,A15)</x:f>
-        <x:v>34</x:v>
+        <x:v>20</x:v>
       </x:c>
     </x:row>
     <x:row r="16">
       <x:c r="A16" t="str">
-        <x:v>Todo (source drift)</x:v>
+        <x:v>Cancelled</x:v>
       </x:c>
       <x:c r="B16" t="n">
-        <x:f>COUNTIF(WBS!$G$4:$G$81,"Todo")</x:f>
-        <x:v>1</x:v>
+        <x:f>COUNTIF(WBS!$G$4:$G$81,A16)</x:f>
+        <x:v>3</x:v>
       </x:c>
     </x:row>
     <x:row r="18">
@@ -2358,7 +2358,7 @@
         <x:v>Freeze prerequisites</x:v>
       </x:c>
       <x:c r="C20" s="13" t="str">
-        <x:v>10/8 goal; capacity before first Freeze. 10/12 proposal not adopted.</x:v>
+        <x:v>#34 Freeze 사양38a6512 확정. actual G4·ROSA·앱 인수는 별도.</x:v>
       </x:c>
       <x:c r="D20" s="195" t="str">
         <x:v>이권욱/이하영/이재환</x:v>
@@ -2372,7 +2372,7 @@
         <x:v>P1 Close</x:v>
       </x:c>
       <x:c r="C21" s="13" t="str">
-        <x:v>#15 endpoint, #16 delivery, #19 rollback unresolved.</x:v>
+        <x:v>모듈·G1~G3 조건부 인수 완료. #31 Review/#30 Signoff/#32 Close 잔여.</x:v>
       </x:c>
       <x:c r="D21" s="195" t="str">
         <x:v>각 P1 Lead</x:v>
@@ -2400,7 +2400,7 @@
         <x:v>D21 evidence</x:v>
       </x:c>
       <x:c r="C23" s="13" t="str">
-        <x:v>Final raw 8706 B; received rehash / publication pending.</x:v>
+        <x:v>D21 확정 사양 편입. 과거 raw intake HOLD를 현재 설계 미결로 사용하지 않음.</x:v>
       </x:c>
       <x:c r="D23" s="195" t="str">
         <x:v>이권욱</x:v>
@@ -2414,7 +2414,7 @@
         <x:v>Source / CA / DNS</x:v>
       </x:c>
       <x:c r="C24" s="13" t="str">
-        <x:v>Model, reconciliation SLA, bilateral DNS and trust pending.</x:v>
+        <x:v>D22 선택A·추가DNS 보류 유지. 실제 CA/Registry/VPN 검증은 각 티켓.</x:v>
       </x:c>
       <x:c r="D24" s="195" t="str">
         <x:v>#34/#38/#42/#47</x:v>
@@ -2428,7 +2428,7 @@
         <x:v>Cost-to-complete</x:v>
       </x:c>
       <x:c r="C25" s="45" t="str">
-        <x:v>Education limit / full resource cost / daily report pending.</x:v>
+        <x:v>기존 예산 경계 유지. 10/19 사용액 보고를 총예상액으로 확대하지 않음.</x:v>
       </x:c>
       <x:c r="D25" s="201" t="str">
         <x:v>이권욱/이하영</x:v>
@@ -2442,7 +2442,7 @@
         <x:v>Same-run evidence</x:v>
       </x:c>
       <x:c r="C26" s="71" t="str">
-        <x:v>Producer #16 / consumer #13; retain 4/4 acceptance.</x:v>
+        <x:v>P1 기존4/4 인수 유지. P2 Runtime은 해당RUN 별도 증적.</x:v>
       </x:c>
       <x:c r="D26" s="202" t="str">
         <x:v>#16/#13</x:v>
@@ -2495,7 +2495,7 @@
     <x:mergeCell ref="A18:V18"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R56581ba0662c47bb"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdb06801cefe24b79"/>
 </x:worksheet>
 </file>
 
@@ -2875,8 +2875,8 @@
           <x:t xml:space="preserve">As of</x:t>
         </x:is>
       </x:c>
-      <x:c r="B2" s="155" t="n">
-        <x:v>46298</x:v>
+      <x:c r="B2" s="155" t="d">
+        <x:v>2026-10-19T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="C2" s="17" t="inlineStr">
         <x:is>
@@ -3062,7 +3062,7 @@
 GitHub closed/completed</x:v>
       </x:c>
       <x:c r="R4" s="13" t="str">
-        <x:v>https://github.com/321Team/fds-project-baseline/issues/7</x:v>
+        <x:v>https://github.com/321Team/fds-project-baseline/issues/7 · 조회 2026-10-19T19:25 KST · body SHA d6e428e32ba8 · 실제종결 2026-09-09T18:39:09+09:00 (completed)</x:v>
       </x:c>
       <x:c r="S4" s="13" t="str">
         <x:f>IF(G4="Done","Done",IF(I4="","End TBD",IF(I4&lt;'Executive Summary'!$B$4,"Target elapsed",IF(H4&gt;'Executive Summary'!$B$4,"Upcoming","Active window"))))</x:f>
@@ -3125,7 +3125,7 @@
 GitHub closed/completed</x:v>
       </x:c>
       <x:c r="R5" s="13" t="str">
-        <x:v>https://github.com/321Team/fds-project-baseline/issues/8</x:v>
+        <x:v>https://github.com/321Team/fds-project-baseline/issues/8 · 조회 2026-10-19T19:25 KST · body SHA 3efc970807fb · 실제종결 2026-09-09T18:40:02+09:00 (completed)</x:v>
       </x:c>
       <x:c r="S5" s="13" t="str">
         <x:f>IF(G5="Done","Done",IF(I5="","End TBD",IF(I5&lt;'Executive Summary'!$B$4,"Target elapsed",IF(H5&gt;'Executive Summary'!$B$4,"Upcoming","Active window"))))</x:f>
@@ -3152,7 +3152,7 @@
         <x:v>P0</x:v>
       </x:c>
       <x:c r="G6" s="13" t="str">
-        <x:v>In Progress</x:v>
+        <x:v>Done</x:v>
       </x:c>
       <x:c r="H6" s="191" t="n">
         <x:v>46261</x:v>
@@ -3188,11 +3188,11 @@
 GitHub open/-</x:v>
       </x:c>
       <x:c r="R6" s="13" t="str">
-        <x:v>https://github.com/321Team/fds-project-baseline/issues/9</x:v>
+        <x:v>https://github.com/321Team/fds-project-baseline/issues/9 · 조회 2026-10-19T19:25 KST · body SHA e2ca980d59d1 · 실제종결 2026-10-05T21:47:24+09:00 (completed)</x:v>
       </x:c>
       <x:c r="S6" s="13" t="str">
         <x:f>IF(G6="Done","Done",IF(I6="","End TBD",IF(I6&lt;'Executive Summary'!$B$4,"Target elapsed",IF(H6&gt;'Executive Summary'!$B$4,"Upcoming","Active window"))))</x:f>
-        <x:v>Target elapsed</x:v>
+        <x:v>Done</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="110" customHeight="1">
@@ -3247,13 +3247,10 @@
         <x:v>LB Stage A 확인, 6개 Node의 보호 공백 없는 firewalld→named HEP/GNP 전환, containerd/kubelet·SELinux·identity·Port Matrix, BGP Disabled+VXLANCrossSubnet Calico, 6/6 Ready, CoreDNS, static local PV Evidence</x:v>
       </x:c>
       <x:c r="Q7" s="195" t="str">
-        <x:v>10/19 조건부 종결. 실제 완료 2026-10-19T18:03:58+09:00. 원 AC/계획일·Owner 보존. 근거 https://github.com/321Team/fds-project-baseline/issues/10#issuecomment-6263610419. 상세 조건은 동봉 Ticket Pack.
-[기존 계획/관측]
-09-11 CP1, 09-14 CP2/3·Worker, 09-15 NTP·Calico, 09-17 증적 인수를 조건부 목표로 둔다. 실제 상태·완료 판정은 유지한다. 세부 배정: Fast Track Plan 시트.
-GitHub open/-</x:v>
+        <x:v>09-11 CP1, 09-14 CP2/3·Worker, 09-15 NTP·Calico, 09-17 증적 인수를 조건부 목표로 둔다. 실제 상태·완료 판정은 유지한다. 세부 배정: Fast Track Plan 시트.</x:v>
       </x:c>
       <x:c r="R7" s="13" t="str">
-        <x:v>https://github.com/321Team/fds-project-baseline/issues/10</x:v>
+        <x:v>https://github.com/321Team/fds-project-baseline/issues/10 · 조회 2026-10-19T19:25 KST · body SHA fb8ece4e98d1 · 실제종결 2026-10-19T18:03:58+09:00 (completed)</x:v>
       </x:c>
       <x:c r="S7" s="13" t="str">
         <x:f>IF(G7="Done","Done",IF(I7="","End TBD",IF(I7&lt;'Executive Summary'!$B$4,"Target elapsed",IF(H7&gt;'Executive Summary'!$B$4,"Upcoming","Active window"))))</x:f>
@@ -3280,7 +3277,7 @@
         <x:v>P0</x:v>
       </x:c>
       <x:c r="G8" s="13" t="str">
-        <x:v>In Progress</x:v>
+        <x:v>Done</x:v>
       </x:c>
       <x:c r="H8" s="191" t="n">
         <x:v>46262</x:v>
@@ -3316,11 +3313,11 @@
 GitHub open/-</x:v>
       </x:c>
       <x:c r="R8" s="13" t="str">
-        <x:v>https://github.com/321Team/fds-project-baseline/issues/11</x:v>
+        <x:v>https://github.com/321Team/fds-project-baseline/issues/11 · 조회 2026-10-19T19:25 KST · body SHA 410534fa4edd · 실제종결 2026-10-14T11:07:34+09:00 (completed)</x:v>
       </x:c>
       <x:c r="S8" s="13" t="str">
         <x:f>IF(G8="Done","Done",IF(I8="","End TBD",IF(I8&lt;'Executive Summary'!$B$4,"Target elapsed",IF(H8&gt;'Executive Summary'!$B$4,"Upcoming","Active window"))))</x:f>
-        <x:v>Target elapsed</x:v>
+        <x:v>Done</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="110" customHeight="1">
@@ -3379,7 +3376,7 @@
 GitHub closed/completed</x:v>
       </x:c>
       <x:c r="R9" s="13" t="str">
-        <x:v>https://github.com/321Team/fds-project-baseline/issues/12</x:v>
+        <x:v>https://github.com/321Team/fds-project-baseline/issues/12 · 조회 2026-10-19T19:25 KST · body SHA 03eb461ade12 · 실제종결 2026-09-09T18:41:10+09:00 (completed)</x:v>
       </x:c>
       <x:c r="S9" s="13" t="str">
         <x:f>IF(G9="Done","Done",IF(I9="","End TBD",IF(I9&lt;'Executive Summary'!$B$4,"Target elapsed",IF(H9&gt;'Executive Summary'!$B$4,"Upcoming","Active window"))))</x:f>
@@ -3438,13 +3435,10 @@
         <x:v>harbor01 `.54:443`, Private CA Trust, 최소권한 Robot Account, IF-09 Runner Push·IF-10 Worker Pull/Pod Start, 비승인 Push/Pull DENY, Trivy/Digest/Evidence PASS</x:v>
       </x:c>
       <x:c r="Q10" s="195" t="str">
-        <x:v>10/19 조건부 종결. 실제 완료 2026-10-19T18:04:15+09:00. 원 AC/계획일·Owner 보존. 근거 https://github.com/321Team/fds-project-baseline/issues/13#issuecomment-6263615041. 상세 조건은 동봉 Ticket Pack.
-[기존 계획/관측]
-Harbor 준비는 CP 후속과 병행하고 09-16 CI Scan Digest까지 4/4 대조 후 09-17 인수 목표다. 실제 상태·완료 판정은 유지한다. 세부 배정: Fast Track Plan 시트.
-GitHub open/-</x:v>
+        <x:v>Harbor 준비는 CP 후속과 병행하고 09-16 CI Scan Digest까지 4/4 대조 후 09-17 인수 목표다. 실제 상태·완료 판정은 유지한다. 세부 배정: Fast Track Plan 시트.</x:v>
       </x:c>
       <x:c r="R10" s="13" t="str">
-        <x:v>https://github.com/321Team/fds-project-baseline/issues/13</x:v>
+        <x:v>https://github.com/321Team/fds-project-baseline/issues/13 · 조회 2026-10-19T19:25 KST · body SHA b70bf46a22d4 · 실제종결 2026-10-19T18:04:15+09:00 (completed)</x:v>
       </x:c>
       <x:c r="S10" s="13" t="str">
         <x:f>IF(G10="Done","Done",IF(I10="","End TBD",IF(I10&lt;'Executive Summary'!$B$4,"Target elapsed",IF(H10&gt;'Executive Summary'!$B$4,"Upcoming","Active window"))))</x:f>
@@ -3503,13 +3497,10 @@
         <x:v>Kubernetes 6개 Node의 보호 공백 없는 firewalld→Calico named HEP/GNP 전환, 30080/9100/10250 최소 허용, 관리망 반환 경로와 IF-06B 정합화, Positive/Negative/Regression/Reboot/Rollback 및 무결성 Evidence 완료</x:v>
       </x:c>
       <x:c r="Q11" s="195" t="str">
-        <x:v>10/19 조건부 인수/판정. 근거 https://github.com/321Team/fds-project-baseline/issues/14#issuecomment-6264595677. 실제 종결 2026-10-19T19:05:24+09:00. 종결 근거 https://github.com/321Team/fds-project-baseline/issues/14#issuecomment-6264705121. 원 AC/계획/Owner와 기술 한계 유지.
-[기존 계획/관측]
-09-21은 권장 Plan End이며 실제 종료일 확정이나 AC 완료가 아니다. 기존 End TBD 이력은 보존한다. CP→Worker·NTP·IF-16을 먼저, IF-06B·Negative/Reboot/Rollback·보호 인계를 후속 검증한다. 실제 상태·완료 판정은 유지한다. 세부 배정: Fast Track Plan 시트.
-GitHub open/-</x:v>
+        <x:v>09-21은 권장 Plan End이며 실제 종료일 확정이나 AC 완료가 아니다. 기존 End TBD 이력은 보존한다. CP→Worker·NTP·IF-16을 먼저, IF-06B·Negative/Reboot/Rollback·보호 인계를 후속 검증한다. 실제 상태·완료 판정은 유지한다. 세부 배정: Fast Track Plan 시트.</x:v>
       </x:c>
       <x:c r="R11" s="13" t="str">
-        <x:v>https://github.com/321Team/fds-project-baseline/issues/14</x:v>
+        <x:v>https://github.com/321Team/fds-project-baseline/issues/14 · 조회 2026-10-19T19:25 KST · body SHA 2da95da77c70 · 실제종결 2026-10-19T19:05:24+09:00 (completed)</x:v>
       </x:c>
       <x:c r="S11" s="13" t="str">
         <x:f>IF(G11="Done","Done",IF(I11="","End TBD",IF(I11&lt;'Executive Summary'!$B$4,"Target elapsed",IF(H11&gt;'Executive Summary'!$B$4,"Upcoming","Active window"))))</x:f>
@@ -3572,7 +3563,7 @@
 GitHub closed/completed</x:v>
       </x:c>
       <x:c r="R12" s="13" t="str">
-        <x:v>https://github.com/321Team/fds-project-baseline/issues/58</x:v>
+        <x:v>https://github.com/321Team/fds-project-baseline/issues/58 · 조회 2026-10-19T19:25 KST · body SHA 871283ea4135 · 실제종결 2026-09-09T18:52:36+09:00 (completed)</x:v>
       </x:c>
       <x:c r="S12" s="13" t="str">
         <x:f>IF(G12="Done","Done",IF(I12="","End TBD",IF(I12&lt;'Executive Summary'!$B$4,"Target elapsed",IF(H12&gt;'Executive Summary'!$B$4,"Upcoming","Active window"))))</x:f>
@@ -3631,14 +3622,10 @@
         <x:v>2개 Deployment/Service, 업무 8000/8001·metrics 9091/9090, `/livez`·`/readyz`, DB/FDS 장애정책, Resource, local endpoint topology, Contract/E2E Evidence</x:v>
       </x:c>
       <x:c r="Q13" s="195" t="str">
-        <x:v>10/19 조건부 종결. 실제 완료 2026-10-19T18:04:23+09:00. 원 AC/계획일·Owner 보존. 근거 https://github.com/321Team/fds-project-baseline/issues/15#issuecomment-6263617401. 상세 조건은 동봉 Ticket Pack.
-[기존 계획/관측]
-09-11 인계 및 사전 검증, 09-18 복귀 후 정본 Runtime 통합. 휴가 중 미승인 업무 계약·Schema 변경은 중단한다. 실제 상태·완료 판정은 유지한다. 세부 배정: Fast Track Plan 시트.
-TS12; local endpoint 보장 NOT MET.
-GitHub open/-</x:v>
+        <x:v>09-11 인계 및 사전 검증, 09-18 복귀 후 정본 Runtime 통합. 휴가 중 미승인 업무 계약·Schema 변경은 중단한다. 실제 상태·완료 판정은 유지한다. 세부 배정: Fast Track Plan 시트.</x:v>
       </x:c>
       <x:c r="R13" s="13" t="str">
-        <x:v>https://github.com/321Team/fds-project-baseline/issues/15</x:v>
+        <x:v>https://github.com/321Team/fds-project-baseline/issues/15 · 조회 2026-10-19T19:25 KST · body SHA 139c96c3100e · 실제종결 2026-10-19T18:04:23+09:00 (completed)</x:v>
       </x:c>
       <x:c r="S13" s="13" t="str">
         <x:f>IF(G13="Done","Done",IF(I13="","End TBD",IF(I13&lt;'Executive Summary'!$B$4,"Target elapsed",IF(H13&gt;'Executive Summary'!$B$4,"Upcoming","Active window"))))</x:f>
@@ -3665,7 +3652,7 @@
         <x:v>P0</x:v>
       </x:c>
       <x:c r="G14" s="13" t="str">
-        <x:v>In Progress</x:v>
+        <x:v>Done</x:v>
       </x:c>
       <x:c r="H14" s="191" t="n">
         <x:v>46266</x:v>
@@ -3702,11 +3689,11 @@
 GitHub open/-</x:v>
       </x:c>
       <x:c r="R14" s="13" t="str">
-        <x:v>https://github.com/321Team/fds-project-baseline/issues/16</x:v>
+        <x:v>https://github.com/321Team/fds-project-baseline/issues/16 · 조회 2026-10-19T19:25 KST · body SHA a67524165c36 · 실제종결 2026-10-15T19:47:58+09:00 (completed)</x:v>
       </x:c>
       <x:c r="S14" s="13" t="str">
         <x:f>IF(G14="Done","Done",IF(I14="","End TBD",IF(I14&lt;'Executive Summary'!$B$4,"Target elapsed",IF(H14&gt;'Executive Summary'!$B$4,"Upcoming","Active window"))))</x:f>
-        <x:v>Target elapsed</x:v>
+        <x:v>Done</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="110" customHeight="1">
@@ -3761,13 +3748,10 @@
         <x:v>Hybrid Monitoring의 Runtime Acceptance 14개와 필수 보조통제 2개, 구축·복구·Rollback Runbook 및 Support Review 증적 확보</x:v>
       </x:c>
       <x:c r="Q15" s="195" t="str">
-        <x:v>10/19 조건부 종결. 실제 완료 2026-10-19T18:04:31+09:00. 원 AC/계획일·Owner 보존. 근거 https://github.com/321Team/fds-project-baseline/issues/17#issuecomment-6263619666. 상세 조건은 동봉 Ticket Pack.
-[기존 계획/관측]
-09-11 Monitoring 인계, 부재 중 기존 Support의 준비·구현, 09-18 복귀 후 14개 AC+2개 보조통제 검증을 목표로 한다. 실제 상태·완료 판정은 유지한다. 세부 배정: Fast Track Plan 시트.
-GitHub open/-</x:v>
+        <x:v>09-11 Monitoring 인계, 부재 중 기존 Support의 준비·구현, 09-18 복귀 후 14개 AC+2개 보조통제 검증을 목표로 한다. 실제 상태·완료 판정은 유지한다. 세부 배정: Fast Track Plan 시트.</x:v>
       </x:c>
       <x:c r="R15" s="13" t="str">
-        <x:v>https://github.com/321Team/fds-project-baseline/issues/17</x:v>
+        <x:v>https://github.com/321Team/fds-project-baseline/issues/17 · 조회 2026-10-19T19:25 KST · body SHA 59e50b43a836 · 실제종결 2026-10-19T18:04:31+09:00 (completed)</x:v>
       </x:c>
       <x:c r="S15" s="13" t="str">
         <x:f>IF(G15="Done","Done",IF(I15="","End TBD",IF(I15&lt;'Executive Summary'!$B$4,"Target elapsed",IF(H15&gt;'Executive Summary'!$B$4,"Upcoming","Active window"))))</x:f>
@@ -3826,13 +3810,10 @@
         <x:v>CentOS/containerd, Ansible Inventory/SSH/멱등성, 3CP+3Worker, API LB/Calico, Harbor/Runner/PostgreSQL, Node Connectivity와 Push/Pull 준비도 승인</x:v>
       </x:c>
       <x:c r="Q16" s="195" t="str">
-        <x:v>10/19 조건부 인수/판정. 근거 https://github.com/321Team/fds-project-baseline/issues/18#issuecomment-6264597081. 실제 종결 2026-10-19T19:05:40+09:00. 종결 근거 https://github.com/321Team/fds-project-baseline/issues/18#issuecomment-6264709975. 원 AC/계획/Owner와 기술 한계 유지.
-[기존 계획/관측]
-09-17 오후 조건부 인수 목표. 6대·API/LB·Calico·DB·Harbor·Runner 증적 미충족이면 PASS 불가. 실제 상태·완료 판정은 유지한다. 세부 배정: Fast Track Plan 시트.
-GitHub open/-</x:v>
+        <x:v>09-17 오후 조건부 인수 목표. 6대·API/LB·Calico·DB·Harbor·Runner 증적 미충족이면 PASS 불가. 실제 상태·완료 판정은 유지한다. 세부 배정: Fast Track Plan 시트.</x:v>
       </x:c>
       <x:c r="R16" s="13" t="str">
-        <x:v>https://github.com/321Team/fds-project-baseline/issues/18</x:v>
+        <x:v>https://github.com/321Team/fds-project-baseline/issues/18 · 조회 2026-10-19T19:25 KST · body SHA 2586f4364edf · 실제종결 2026-10-19T19:05:40+09:00 (completed)</x:v>
       </x:c>
       <x:c r="S16" s="13" t="str">
         <x:f>IF(G16="Done","Done",IF(I16="","End TBD",IF(I16&lt;'Executive Summary'!$B$4,"Target elapsed",IF(H16&gt;'Executive Summary'!$B$4,"Upcoming","Active window"))))</x:f>
@@ -3891,14 +3872,10 @@
         <x:v>PSA/SecurityContext/Default Deny/RBAC/HEP-GNP/Secretbox/LimitRange/Probe와 `.50/32→30080` 포함 Positive·Negative·Rollback Evidence PASS</x:v>
       </x:c>
       <x:c r="Q17" s="195" t="str">
-        <x:v>10/19 조건부 종결. 실제 완료 2026-10-19T18:04:07+09:00. 원 AC/계획일·Owner 보존. 근거 https://github.com/321Team/fds-project-baseline/issues/19#issuecomment-6263612875. 상세 조건은 동봉 Ticket Pack.
-[기존 계획/관측]
-09-10 휴가 추가 후 기존 09-04~11 가용일은 4일. 권장 종료 09-21로 확장한 전체 계획창의 가용일은 10일이며 잔여 공수를 뜻하지 않는다. Runtime 검증은 플랫폼·앱 인수와 연계한다. 실제 상태·완료 판정은 유지한다. 세부 배정: Fast Track Plan 시트.
-TS13; rollback 4 blockers / 변경창 HOLD. rotation NOT MET/RISK ACCEPTED.
-GitHub open/-</x:v>
+        <x:v>09-10 휴가 추가 후 기존 09-04~11 가용일은 4일. 권장 종료 09-21로 확장한 전체 계획창의 가용일은 10일이며 잔여 공수를 뜻하지 않는다. Runtime 검증은 플랫폼·앱 인수와 연계한다. 실제 상태·완료 판정은 유지한다. 세부 배정: Fast Track Plan 시트.</x:v>
       </x:c>
       <x:c r="R17" s="13" t="str">
-        <x:v>https://github.com/321Team/fds-project-baseline/issues/19</x:v>
+        <x:v>https://github.com/321Team/fds-project-baseline/issues/19 · 조회 2026-10-19T19:25 KST · body SHA 04ff69e4cc83 · 실제종결 2026-10-19T18:04:07+09:00 (completed)</x:v>
       </x:c>
       <x:c r="S17" s="13" t="str">
         <x:f>IF(G17="Done","Done",IF(I17="","End TBD",IF(I17&lt;'Executive Summary'!$B$4,"Target elapsed",IF(H17&gt;'Executive Summary'!$B$4,"Upcoming","Active window"))))</x:f>
@@ -3957,13 +3934,10 @@
         <x:v>Client→edge→transaction-api→fds-engine→PostgreSQL→Prometheus E2E, Rule·Negative·Regression PASS, Critical Issue 0 및 Evidence 승인</x:v>
       </x:c>
       <x:c r="Q18" s="195" t="str">
-        <x:v>10/19 조건부 종결. 실제 완료 2026-10-19T18:04:40+09:00. 원 AC/계획일·Owner 보존. 근거 https://github.com/321Team/fds-project-baseline/issues/20#issuecomment-6263622038. 상세 조건은 동봉 Ticket Pack.
-[기존 계획/관측]
-10-05 공휴일/비근무를 반영해 Phase 1 최종 Runtime 회귀·증적 보강 목표를 10-02(금)로 고정한다. 10-06은 Review/Close 전용이며 신규 대규모 구현을 배정하지 않는다.
-GitHub open/-</x:v>
+        <x:v>10-05 공휴일/비근무를 반영해 Phase 1 최종 Runtime 회귀·증적 보강 목표를 10-02(금)로 고정한다. 10-06은 Review/Close 전용이며 신규 대규모 구현을 배정하지 않는다.</x:v>
       </x:c>
       <x:c r="R18" s="13" t="str">
-        <x:v>https://github.com/321Team/fds-project-baseline/issues/20</x:v>
+        <x:v>https://github.com/321Team/fds-project-baseline/issues/20 · 조회 2026-10-19T19:25 KST · body SHA 71009256c529 · 실제종결 2026-10-19T18:04:40+09:00 (completed)</x:v>
       </x:c>
       <x:c r="S18" s="13" t="str">
         <x:f>IF(G18="Done","Done",IF(I18="","End TBD",IF(I18&lt;'Executive Summary'!$B$4,"Target elapsed",IF(H18&gt;'Executive Summary'!$B$4,"Upcoming","Active window"))))</x:f>
@@ -3990,7 +3964,7 @@
         <x:v>P0</x:v>
       </x:c>
       <x:c r="G19" s="13" t="str">
-        <x:v>In Progress</x:v>
+        <x:v>Done</x:v>
       </x:c>
       <x:c r="H19" s="191" t="n">
         <x:v>46276</x:v>
@@ -4026,11 +4000,11 @@
 GitHub open/-</x:v>
       </x:c>
       <x:c r="R19" s="13" t="str">
-        <x:v>https://github.com/321Team/fds-project-baseline/issues/21</x:v>
+        <x:v>https://github.com/321Team/fds-project-baseline/issues/21 · 조회 2026-10-19T19:25 KST · body SHA eb16fbacd6ad · 실제종결 2026-10-13T13:46:59+09:00 (completed)</x:v>
       </x:c>
       <x:c r="S19" s="13" t="str">
         <x:f>IF(G19="Done","Done",IF(I19="","End TBD",IF(I19&lt;'Executive Summary'!$B$4,"Target elapsed",IF(H19&gt;'Executive Summary'!$B$4,"Upcoming","Active window"))))</x:f>
-        <x:v>Target elapsed</x:v>
+        <x:v>Done</x:v>
       </x:c>
     </x:row>
     <x:row r="20" ht="110" customHeight="1">
@@ -4053,7 +4027,7 @@
         <x:v>P0</x:v>
       </x:c>
       <x:c r="G20" s="13" t="str">
-        <x:v>In Progress</x:v>
+        <x:v>Done</x:v>
       </x:c>
       <x:c r="H20" s="191" t="n">
         <x:v>46276</x:v>
@@ -4089,11 +4063,11 @@
 GitHub open/-</x:v>
       </x:c>
       <x:c r="R20" s="13" t="str">
-        <x:v>https://github.com/321Team/fds-project-baseline/issues/22</x:v>
+        <x:v>https://github.com/321Team/fds-project-baseline/issues/22 · 조회 2026-10-19T19:25 KST · body SHA f6d54730794b · 실제종결 2026-10-18T05:05:16+09:00 (completed)</x:v>
       </x:c>
       <x:c r="S20" s="13" t="str">
         <x:f>IF(G20="Done","Done",IF(I20="","End TBD",IF(I20&lt;'Executive Summary'!$B$4,"Target elapsed",IF(H20&gt;'Executive Summary'!$B$4,"Upcoming","Active window"))))</x:f>
-        <x:v>Target elapsed</x:v>
+        <x:v>Done</x:v>
       </x:c>
     </x:row>
     <x:row r="21" ht="110" customHeight="1">
@@ -4148,13 +4122,10 @@
         <x:v>2-Service MSA, DB 저장, Security P0, CI/CD, Monitoring, Initial E2E/Negative Test/Worker Drain 준비도를 승인</x:v>
       </x:c>
       <x:c r="Q21" s="195" t="str">
-        <x:v>10/19 조건부 인수/판정. 근거 https://github.com/321Team/fds-project-baseline/issues/23#issuecomment-6264221185. 실제 종결 2026-10-19T19:05:48+09:00. 종결 근거 https://github.com/321Team/fds-project-baseline/issues/23#issuecomment-6264712221. 원 AC/계획/Owner와 기술 한계 유지.
-[기존 계획/관측]
-09-21 오후 종료 시점 목표. 앱/보안/CI/Monitoring·초기 E2E/Negative/Drain 준비도와 해당 증적이 선행한다. 실제 상태·완료 판정은 유지한다. 세부 배정: Fast Track Plan 시트.
-GitHub open/-</x:v>
+        <x:v>09-21 오후 종료 시점 목표. 앱/보안/CI/Monitoring·초기 E2E/Negative/Drain 준비도와 해당 증적이 선행한다. 실제 상태·완료 판정은 유지한다. 세부 배정: Fast Track Plan 시트.</x:v>
       </x:c>
       <x:c r="R21" s="13" t="str">
-        <x:v>https://github.com/321Team/fds-project-baseline/issues/23</x:v>
+        <x:v>https://github.com/321Team/fds-project-baseline/issues/23 · 조회 2026-10-19T19:25 KST · body SHA cd8820fb19c0 · 실제종결 2026-10-19T19:05:48+09:00 (completed)</x:v>
       </x:c>
       <x:c r="S21" s="13" t="str">
         <x:f>IF(G21="Done","Done",IF(I21="","End TBD",IF(I21&lt;'Executive Summary'!$B$4,"Target elapsed",IF(H21&gt;'Executive Summary'!$B$4,"Upcoming","Active window"))))</x:f>
@@ -4213,13 +4184,10 @@
         <x:v>As-built Architecture, Test/Evidence Index, 구축·운영·복구 Runbook, P1 미완료 Known Issue의 풀네임 Owner·Due, Version/Source 및 Review 재현성 승인</x:v>
       </x:c>
       <x:c r="Q22" s="195" t="str">
-        <x:v>10/19 조건부 종결. 실제 완료 2026-10-19T18:12:54+09:00. 원 AC/계획일·Owner 보존. 근거 https://github.com/321Team/fds-project-baseline/issues/24#issuecomment-6263765512. 상세 조건은 동봉 Ticket Pack.
-[기존 계획/관측]
-Phase 1 Review package 동결 목표를 10-02(금)로 조정한다. 10-05는 비근무일, 10-06은 Review/Close 전용이다. Source/Evidence 미완료는 Known Issue 또는 잔여 Action으로 명시한다.
-GitHub open/-</x:v>
+        <x:v>Phase 1 Review package 동결 목표를 10-02(금)로 조정한다. 10-05는 비근무일, 10-06은 Review/Close 전용이다. Source/Evidence 미완료는 Known Issue 또는 잔여 Action으로 명시한다.</x:v>
       </x:c>
       <x:c r="R22" s="13" t="str">
-        <x:v>https://github.com/321Team/fds-project-baseline/issues/24</x:v>
+        <x:v>https://github.com/321Team/fds-project-baseline/issues/24 · 조회 2026-10-19T19:25 KST · body SHA cf96de6b835a · 실제종결 2026-10-19T18:12:54+09:00 (completed)</x:v>
       </x:c>
       <x:c r="S22" s="13" t="str">
         <x:f>IF(G22="Done","Done",IF(I22="","End TBD",IF(I22&lt;'Executive Summary'!$B$4,"Target elapsed",IF(H22&gt;'Executive Summary'!$B$4,"Upcoming","Active window"))))</x:f>
@@ -4234,7 +4202,7 @@
         <x:v>Dashboard / Alert Enhancement</x:v>
       </x:c>
       <x:c r="C23" s="13" t="str">
-        <x:v>Phase 1</x:v>
+        <x:v>Phase 2</x:v>
       </x:c>
       <x:c r="D23" s="13" t="str">
         <x:v>Monitoring / Observability</x:v>
@@ -4277,7 +4245,7 @@
 원문 일정: TBD — P0 인수 후 재계획 / TBD — 구현 유예 권장</x:v>
       </x:c>
       <x:c r="R23" s="13" t="str">
-        <x:v>https://github.com/321Team/fds-project-baseline/issues/25</x:v>
+        <x:v>https://github.com/321Team/fds-project-baseline/issues/25 · 조회 2026-10-19T19:25 KST · body SHA 1e1ce4b45278</x:v>
       </x:c>
       <x:c r="S23" s="13" t="str">
         <x:f>IF(G23="Done","Done",IF(I23="","End TBD",IF(I23&lt;'Executive Summary'!$B$4,"Target elapsed",IF(H23&gt;'Executive Summary'!$B$4,"Upcoming","Active window"))))</x:f>
@@ -4292,7 +4260,7 @@
         <x:v>Harbor / etcd Backup and Restore</x:v>
       </x:c>
       <x:c r="C24" s="13" t="str">
-        <x:v>Phase 1</x:v>
+        <x:v>Phase 2</x:v>
       </x:c>
       <x:c r="D24" s="13" t="str">
         <x:v>DR / Platform Recovery</x:v>
@@ -4335,7 +4303,7 @@
 원문 일정: TBD — P0 인수 후 재계획 / TBD — 구현 유예 권장</x:v>
       </x:c>
       <x:c r="R24" s="13" t="str">
-        <x:v>https://github.com/321Team/fds-project-baseline/issues/26</x:v>
+        <x:v>https://github.com/321Team/fds-project-baseline/issues/26 · 조회 2026-10-19T19:25 KST · body SHA 29da57d4e92b</x:v>
       </x:c>
       <x:c r="S24" s="13" t="str">
         <x:f>IF(G24="Done","Done",IF(I24="","End TBD",IF(I24&lt;'Executive Summary'!$B$4,"Target elapsed",IF(H24&gt;'Executive Summary'!$B$4,"Upcoming","Active window"))))</x:f>
@@ -4350,7 +4318,7 @@
         <x:v>Platform Resilience P1 Validation</x:v>
       </x:c>
       <x:c r="C25" s="13" t="str">
-        <x:v>Phase 1</x:v>
+        <x:v>Phase 2</x:v>
       </x:c>
       <x:c r="D25" s="13" t="str">
         <x:v>HA / Platform Resilience</x:v>
@@ -4393,7 +4361,7 @@
 원문 일정: TBD — P0 인수 후 재계획 / TBD — 구현 유예 권장</x:v>
       </x:c>
       <x:c r="R25" s="13" t="str">
-        <x:v>https://github.com/321Team/fds-project-baseline/issues/27</x:v>
+        <x:v>https://github.com/321Team/fds-project-baseline/issues/27 · 조회 2026-10-19T19:25 KST · body SHA e052bb42c701</x:v>
       </x:c>
       <x:c r="S25" s="13" t="str">
         <x:f>IF(G25="Done","Done",IF(I25="","End TBD",IF(I25&lt;'Executive Summary'!$B$4,"Target elapsed",IF(H25&gt;'Executive Summary'!$B$4,"Upcoming","Active window"))))</x:f>
@@ -4456,7 +4424,7 @@
 GitHub closed/completed</x:v>
       </x:c>
       <x:c r="R26" s="13" t="str">
-        <x:v>https://github.com/321Team/fds-project-baseline/issues/28</x:v>
+        <x:v>https://github.com/321Team/fds-project-baseline/issues/28 · 조회 2026-10-19T19:25 KST · body SHA baaa15a37335 · 실제종결 2026-09-16T17:53:19+09:00 (completed)</x:v>
       </x:c>
       <x:c r="S26" s="13" t="str">
         <x:f>IF(G26="Done","Done",IF(I26="","End TBD",IF(I26&lt;'Executive Summary'!$B$4,"Target elapsed",IF(H26&gt;'Executive Summary'!$B$4,"Upcoming","Active window"))))</x:f>
@@ -4515,13 +4483,10 @@
         <x:v>Final E2E/Regression, Worker Drain, PostgreSQL Restore, Critical Issue 0, Architecture/Test/Runbook 준비도를 승인</x:v>
       </x:c>
       <x:c r="Q27" s="195" t="str">
-        <x:v>10/19 조건부 인수/판정. 근거 https://github.com/321Team/fds-project-baseline/issues/29#issuecomment-6264597709. 실제 종결 2026-10-19T19:05:55+09:00. 종결 근거 https://github.com/321Team/fds-project-baseline/issues/29#issuecomment-6264714186. 원 AC/계획/Owner와 기술 한계 유지.
-[기존 계획/관측]
-10-02는 실작업·증적 cutoff/G3 Review Ready 판정일이다. 남은 Phase 1 P0는 담당자별 공유 Runtime으로 직렬화하고, 미완료 AC는 10-06 Review에서 사실 상태를 분류한다. 일정 도래만으로 Gate PASS 처리하지 않는다.
-GitHub open/-</x:v>
+        <x:v>10-02는 실작업·증적 cutoff/G3 Review Ready 판정일이다. 남은 Phase 1 P0는 담당자별 공유 Runtime으로 직렬화하고, 미완료 AC는 10-06 Review에서 사실 상태를 분류한다. 일정 도래만으로 Gate PASS 처리하지 않는다.</x:v>
       </x:c>
       <x:c r="R27" s="13" t="str">
-        <x:v>https://github.com/321Team/fds-project-baseline/issues/29</x:v>
+        <x:v>https://github.com/321Team/fds-project-baseline/issues/29 · 조회 2026-10-19T19:25 KST · body SHA 33376af922bc · 실제종결 2026-10-19T19:05:55+09:00 (completed)</x:v>
       </x:c>
       <x:c r="S27" s="13" t="str">
         <x:f>IF(G27="Done","Done",IF(I27="","End TBD",IF(I27&lt;'Executive Summary'!$B$4,"Target elapsed",IF(H27&gt;'Executive Summary'!$B$4,"Upcoming","Active window"))))</x:f>
@@ -4548,7 +4513,7 @@
         <x:v>P0</x:v>
       </x:c>
       <x:c r="G28" s="13" t="str">
-        <x:v>To Do</x:v>
+        <x:v>In Progress</x:v>
       </x:c>
       <x:c r="H28" s="191" t="n">
         <x:v>46301</x:v>
@@ -4585,11 +4550,11 @@
 GitHub open/-</x:v>
       </x:c>
       <x:c r="R28" s="13" t="str">
-        <x:v>https://github.com/321Team/fds-project-baseline/issues/30</x:v>
+        <x:v>https://github.com/321Team/fds-project-baseline/issues/30 · 조회 2026-10-19T19:25 KST · body SHA adae54557399</x:v>
       </x:c>
       <x:c r="S28" s="13" t="str">
         <x:f>IF(G28="Done","Done",IF(I28="","End TBD",IF(I28&lt;'Executive Summary'!$B$4,"Target elapsed",IF(H28&gt;'Executive Summary'!$B$4,"Upcoming","Active window"))))</x:f>
-        <x:v>Upcoming</x:v>
+        <x:v>Target elapsed</x:v>
       </x:c>
     </x:row>
     <x:row r="29" ht="110" customHeight="1">
@@ -4612,7 +4577,7 @@
         <x:v>P0</x:v>
       </x:c>
       <x:c r="G29" s="13" t="str">
-        <x:v>To Do</x:v>
+        <x:v>In Progress</x:v>
       </x:c>
       <x:c r="H29" s="191" t="n">
         <x:v>46301</x:v>
@@ -4648,11 +4613,11 @@
 GitHub open/-</x:v>
       </x:c>
       <x:c r="R29" s="13" t="str">
-        <x:v>https://github.com/321Team/fds-project-baseline/issues/31</x:v>
+        <x:v>https://github.com/321Team/fds-project-baseline/issues/31 · 조회 2026-10-19T19:25 KST · body SHA 7b0b4bb69e61</x:v>
       </x:c>
       <x:c r="S29" s="13" t="str">
         <x:f>IF(G29="Done","Done",IF(I29="","End TBD",IF(I29&lt;'Executive Summary'!$B$4,"Target elapsed",IF(H29&gt;'Executive Summary'!$B$4,"Upcoming","Active window"))))</x:f>
-        <x:v>Upcoming</x:v>
+        <x:v>Target elapsed</x:v>
       </x:c>
     </x:row>
     <x:row r="30" ht="110" customHeight="1">
@@ -4711,11 +4676,11 @@
 GitHub open/-</x:v>
       </x:c>
       <x:c r="R30" s="13" t="str">
-        <x:v>https://github.com/321Team/fds-project-baseline/issues/32</x:v>
+        <x:v>https://github.com/321Team/fds-project-baseline/issues/32 · 조회 2026-10-19T19:25 KST · body SHA be9aebeff65a</x:v>
       </x:c>
       <x:c r="S30" s="13" t="str">
         <x:f>IF(G30="Done","Done",IF(I30="","End TBD",IF(I30&lt;'Executive Summary'!$B$4,"Target elapsed",IF(H30&gt;'Executive Summary'!$B$4,"Upcoming","Active window"))))</x:f>
-        <x:v>Upcoming</x:v>
+        <x:v>Target elapsed</x:v>
       </x:c>
     </x:row>
     <x:row r="31" ht="110" customHeight="1">
@@ -4774,11 +4739,11 @@
 GitHub open/-</x:v>
       </x:c>
       <x:c r="R31" s="13" t="str">
-        <x:v>https://github.com/321Team/fds-project-baseline/issues/33</x:v>
+        <x:v>https://github.com/321Team/fds-project-baseline/issues/33 · 조회 2026-10-19T19:25 KST · body SHA d3b53a69ea62</x:v>
       </x:c>
       <x:c r="S31" s="13" t="str">
         <x:f>IF(G31="Done","Done",IF(I31="","End TBD",IF(I31&lt;'Executive Summary'!$B$4,"Target elapsed",IF(H31&gt;'Executive Summary'!$B$4,"Upcoming","Active window"))))</x:f>
-        <x:v>Upcoming</x:v>
+        <x:v>Target elapsed</x:v>
       </x:c>
     </x:row>
     <x:row r="32" ht="110" customHeight="1">
@@ -4801,7 +4766,7 @@
         <x:v>P0</x:v>
       </x:c>
       <x:c r="G32" s="13" t="str">
-        <x:v>To Do</x:v>
+        <x:v>Done</x:v>
       </x:c>
       <x:c r="H32" s="191" t="n">
         <x:v>46303</x:v>
@@ -4838,11 +4803,11 @@
 GitHub open/-</x:v>
       </x:c>
       <x:c r="R32" s="13" t="str">
-        <x:v>https://github.com/321Team/fds-project-baseline/issues/34</x:v>
+        <x:v>https://github.com/321Team/fds-project-baseline/issues/34 · 조회 2026-10-19T19:25 KST · body SHA 2dbc6ac6e298 · 실제종결 2026-10-19T18:38:16+09:00 (completed)</x:v>
       </x:c>
       <x:c r="S32" s="13" t="str">
         <x:f>IF(G32="Done","Done",IF(I32="","End TBD",IF(I32&lt;'Executive Summary'!$B$4,"Target elapsed",IF(H32&gt;'Executive Summary'!$B$4,"Upcoming","Active window"))))</x:f>
-        <x:v>Upcoming</x:v>
+        <x:v>Done</x:v>
       </x:c>
     </x:row>
     <x:row r="33" ht="110" customHeight="1">
@@ -4865,7 +4830,7 @@
         <x:v>P0</x:v>
       </x:c>
       <x:c r="G33" s="13" t="str">
-        <x:v>To Do</x:v>
+        <x:v>In Progress</x:v>
       </x:c>
       <x:c r="H33" s="191" t="n">
         <x:v>46303</x:v>
@@ -4902,11 +4867,11 @@
 GitHub open/-</x:v>
       </x:c>
       <x:c r="R33" s="13" t="str">
-        <x:v>https://github.com/321Team/fds-project-baseline/issues/35</x:v>
+        <x:v>https://github.com/321Team/fds-project-baseline/issues/35 · 조회 2026-10-19T19:25 KST · body SHA 677720e9b9fc</x:v>
       </x:c>
       <x:c r="S33" s="13" t="str">
         <x:f>IF(G33="Done","Done",IF(I33="","End TBD",IF(I33&lt;'Executive Summary'!$B$4,"Target elapsed",IF(H33&gt;'Executive Summary'!$B$4,"Upcoming","Active window"))))</x:f>
-        <x:v>Upcoming</x:v>
+        <x:v>Target elapsed</x:v>
       </x:c>
     </x:row>
     <x:row r="34" ht="110" customHeight="1">
@@ -4929,7 +4894,7 @@
         <x:v>P0</x:v>
       </x:c>
       <x:c r="G34" s="13" t="str">
-        <x:v>To Do</x:v>
+        <x:v>In Progress</x:v>
       </x:c>
       <x:c r="H34" s="191" t="n">
         <x:v>46302</x:v>
@@ -4966,11 +4931,11 @@
 GitHub open/-</x:v>
       </x:c>
       <x:c r="R34" s="13" t="str">
-        <x:v>https://github.com/321Team/fds-project-baseline/issues/36</x:v>
+        <x:v>https://github.com/321Team/fds-project-baseline/issues/36 · 조회 2026-10-19T19:25 KST · body SHA f70908ecded8</x:v>
       </x:c>
       <x:c r="S34" s="13" t="str">
         <x:f>IF(G34="Done","Done",IF(I34="","End TBD",IF(I34&lt;'Executive Summary'!$B$4,"Target elapsed",IF(H34&gt;'Executive Summary'!$B$4,"Upcoming","Active window"))))</x:f>
-        <x:v>Upcoming</x:v>
+        <x:v>Target elapsed</x:v>
       </x:c>
     </x:row>
     <x:row r="35" ht="110" customHeight="1">
@@ -4993,7 +4958,7 @@
         <x:v>P0</x:v>
       </x:c>
       <x:c r="G35" s="13" t="str">
-        <x:v>To Do</x:v>
+        <x:v>In Progress</x:v>
       </x:c>
       <x:c r="H35" s="191" t="n">
         <x:v>46307</x:v>
@@ -5030,11 +4995,11 @@
 GitHub open/-</x:v>
       </x:c>
       <x:c r="R35" s="13" t="str">
-        <x:v>https://github.com/321Team/fds-project-baseline/issues/37</x:v>
+        <x:v>https://github.com/321Team/fds-project-baseline/issues/37 · 조회 2026-10-19T19:25 KST · body SHA 2b32f927a8fe</x:v>
       </x:c>
       <x:c r="S35" s="13" t="str">
         <x:f>IF(G35="Done","Done",IF(I35="","End TBD",IF(I35&lt;'Executive Summary'!$B$4,"Target elapsed",IF(H35&gt;'Executive Summary'!$B$4,"Upcoming","Active window"))))</x:f>
-        <x:v>Upcoming</x:v>
+        <x:v>Target elapsed</x:v>
       </x:c>
     </x:row>
     <x:row r="36" ht="110" customHeight="1">
@@ -5057,7 +5022,7 @@
         <x:v>P0</x:v>
       </x:c>
       <x:c r="G36" s="13" t="str">
-        <x:v>To Do</x:v>
+        <x:v>In Progress</x:v>
       </x:c>
       <x:c r="H36" s="191" t="n">
         <x:v>46310</x:v>
@@ -5094,11 +5059,11 @@
 GitHub open/-</x:v>
       </x:c>
       <x:c r="R36" s="13" t="str">
-        <x:v>https://github.com/321Team/fds-project-baseline/issues/38</x:v>
+        <x:v>https://github.com/321Team/fds-project-baseline/issues/38 · 조회 2026-10-19T19:25 KST · body SHA 525d74d322a0</x:v>
       </x:c>
       <x:c r="S36" s="13" t="str">
         <x:f>IF(G36="Done","Done",IF(I36="","End TBD",IF(I36&lt;'Executive Summary'!$B$4,"Target elapsed",IF(H36&gt;'Executive Summary'!$B$4,"Upcoming","Active window"))))</x:f>
-        <x:v>Upcoming</x:v>
+        <x:v>Active window</x:v>
       </x:c>
     </x:row>
     <x:row r="37" ht="110" customHeight="1">
@@ -5157,11 +5122,11 @@
 GitHub open/-</x:v>
       </x:c>
       <x:c r="R37" s="13" t="str">
-        <x:v>https://github.com/321Team/fds-project-baseline/issues/39</x:v>
+        <x:v>https://github.com/321Team/fds-project-baseline/issues/39 · 조회 2026-10-19T19:25 KST · body SHA da58acabefb5</x:v>
       </x:c>
       <x:c r="S37" s="13" t="str">
         <x:f>IF(G37="Done","Done",IF(I37="","End TBD",IF(I37&lt;'Executive Summary'!$B$4,"Target elapsed",IF(H37&gt;'Executive Summary'!$B$4,"Upcoming","Active window"))))</x:f>
-        <x:v>Upcoming</x:v>
+        <x:v>Target elapsed</x:v>
       </x:c>
     </x:row>
     <x:row r="38" ht="110" customHeight="1">
@@ -5216,16 +5181,14 @@
         <x:v>P0 IP Endpoint 유지 또는 Hybrid DNS P1 적용을 확정하고 Resolver/Forwarding/Zone/Route/테스트·Cancelled 결정 근거를 승인</x:v>
       </x:c>
       <x:c r="Q38" s="195" t="str">
-        <x:v>P0 Hybrid 경로 차단을 피하기 위해 10-16 단일 Decision window에서 IP Endpoint 유지 또는 DNS P1 적용을 확정한다. 구현(#48)은 Go이면서 P0 잔여 capacity가 있을 때만 별도 착수한다.
-TS04; 전체 P1 유지. private 필수 DNS subset은 pre-create 계약.
-GitHub open/-</x:v>
+        <x:v>보류(Deferred) — 2026-10-14 이권욱 결정. D23 추가 Hybrid DNS 도입 보류 확정; 기존 DB/Harbor IP 및 ROSA public API/Route DNS·엄격 TLS 기준 유지. Owner 이권욱. 기존10/16은 보류 재검토 기준일이며 자동 재개 승인이 아니다. 재개는 이권욱의 별도 판단 후 결정. 기존 계획 기준: P0 Hybrid 경로 차단을 피하기 위해 10-16 단일 Decision window에서 IP Endpoint 유지 또는 DNS P1 적용을 확정한다. 구현(#48)은 Go이면서 P0 잔여 capacity가 있을 때만 별도 착수한다.</x:v>
       </x:c>
       <x:c r="R38" s="13" t="str">
-        <x:v>https://github.com/321Team/fds-project-baseline/issues/40</x:v>
+        <x:v>https://github.com/321Team/fds-project-baseline/issues/40 · 조회 2026-10-19T19:25 KST · body SHA 40ce4afdd023</x:v>
       </x:c>
       <x:c r="S38" s="13" t="str">
         <x:f>IF(G38="Done","Done",IF(I38="","End TBD",IF(I38&lt;'Executive Summary'!$B$4,"Target elapsed",IF(H38&gt;'Executive Summary'!$B$4,"Upcoming","Active window"))))</x:f>
-        <x:v>Upcoming</x:v>
+        <x:v>Target elapsed</x:v>
       </x:c>
     </x:row>
     <x:row r="39" ht="110" customHeight="1">
@@ -5279,7 +5242,7 @@
 원문 일정: TBD — G5 이후 P0 잔여 capacity 시 / TBD — 10-26 이전 강제하지 않음</x:v>
       </x:c>
       <x:c r="R39" s="13" t="str">
-        <x:v>https://github.com/321Team/fds-project-baseline/issues/41</x:v>
+        <x:v>https://github.com/321Team/fds-project-baseline/issues/41 · 조회 2026-10-19T19:25 KST · body SHA 70621b661bde</x:v>
       </x:c>
       <x:c r="S39" s="13" t="str">
         <x:f>IF(G39="Done","Done",IF(I39="","End TBD",IF(I39&lt;'Executive Summary'!$B$4,"Target elapsed",IF(H39&gt;'Executive Summary'!$B$4,"Upcoming","Active window"))))</x:f>
@@ -5306,7 +5269,7 @@
         <x:v>P0</x:v>
       </x:c>
       <x:c r="G40" s="13" t="str">
-        <x:v>To Do</x:v>
+        <x:v>In Progress</x:v>
       </x:c>
       <x:c r="H40" s="191" t="n">
         <x:v>46310</x:v>
@@ -5343,11 +5306,11 @@
 GitHub open/-</x:v>
       </x:c>
       <x:c r="R40" s="13" t="str">
-        <x:v>https://github.com/321Team/fds-project-baseline/issues/42</x:v>
+        <x:v>https://github.com/321Team/fds-project-baseline/issues/42 · 조회 2026-10-19T19:25 KST · body SHA 56c124765e65</x:v>
       </x:c>
       <x:c r="S40" s="13" t="str">
         <x:f>IF(G40="Done","Done",IF(I40="","End TBD",IF(I40&lt;'Executive Summary'!$B$4,"Target elapsed",IF(H40&gt;'Executive Summary'!$B$4,"Upcoming","Active window"))))</x:f>
-        <x:v>Upcoming</x:v>
+        <x:v>Target elapsed</x:v>
       </x:c>
     </x:row>
     <x:row r="41" ht="110" customHeight="1">
@@ -5370,7 +5333,7 @@
         <x:v>P0</x:v>
       </x:c>
       <x:c r="G41" s="13" t="str">
-        <x:v>To Do</x:v>
+        <x:v>In Progress</x:v>
       </x:c>
       <x:c r="H41" s="191" t="n">
         <x:v>46311</x:v>
@@ -5407,11 +5370,11 @@
 GitHub open/-</x:v>
       </x:c>
       <x:c r="R41" s="13" t="str">
-        <x:v>https://github.com/321Team/fds-project-baseline/issues/43</x:v>
+        <x:v>https://github.com/321Team/fds-project-baseline/issues/43 · 조회 2026-10-19T19:25 KST · body SHA 449a971a44a4</x:v>
       </x:c>
       <x:c r="S41" s="13" t="str">
         <x:f>IF(G41="Done","Done",IF(I41="","End TBD",IF(I41&lt;'Executive Summary'!$B$4,"Target elapsed",IF(H41&gt;'Executive Summary'!$B$4,"Upcoming","Active window"))))</x:f>
-        <x:v>Upcoming</x:v>
+        <x:v>Active window</x:v>
       </x:c>
     </x:row>
     <x:row r="42" ht="110" customHeight="1">
@@ -5465,7 +5428,7 @@
 원문 일정: TBD — G5 이후 P0 잔여 capacity 시 / TBD — 10-26 이전 강제하지 않음</x:v>
       </x:c>
       <x:c r="R42" s="13" t="str">
-        <x:v>https://github.com/321Team/fds-project-baseline/issues/44</x:v>
+        <x:v>https://github.com/321Team/fds-project-baseline/issues/44 · 조회 2026-10-19T19:25 KST · body SHA 1cee52911729</x:v>
       </x:c>
       <x:c r="S42" s="13" t="str">
         <x:f>IF(G42="Done","Done",IF(I42="","End TBD",IF(I42&lt;'Executive Summary'!$B$4,"Target elapsed",IF(H42&gt;'Executive Summary'!$B$4,"Upcoming","Active window"))))</x:f>
@@ -5528,7 +5491,7 @@
 GitHub open/-</x:v>
       </x:c>
       <x:c r="R43" s="13" t="str">
-        <x:v>https://github.com/321Team/fds-project-baseline/issues/45</x:v>
+        <x:v>https://github.com/321Team/fds-project-baseline/issues/45 · 조회 2026-10-19T19:25 KST · body SHA 3b700affe8cb</x:v>
       </x:c>
       <x:c r="S43" s="13" t="str">
         <x:f>IF(G43="Done","Done",IF(I43="","End TBD",IF(I43&lt;'Executive Summary'!$B$4,"Target elapsed",IF(H43&gt;'Executive Summary'!$B$4,"Upcoming","Active window"))))</x:f>
@@ -5555,7 +5518,7 @@
         <x:v>P0</x:v>
       </x:c>
       <x:c r="G44" s="13" t="str">
-        <x:v>To Do</x:v>
+        <x:v>In Progress</x:v>
       </x:c>
       <x:c r="H44" s="191" t="n">
         <x:v>46315</x:v>
@@ -5592,7 +5555,7 @@
 GitHub open/-</x:v>
       </x:c>
       <x:c r="R44" s="13" t="str">
-        <x:v>https://github.com/321Team/fds-project-baseline/issues/46</x:v>
+        <x:v>https://github.com/321Team/fds-project-baseline/issues/46 · 조회 2026-10-19T19:25 KST · body SHA 071fdb0ed2a2</x:v>
       </x:c>
       <x:c r="S44" s="13" t="str">
         <x:f>IF(G44="Done","Done",IF(I44="","End TBD",IF(I44&lt;'Executive Summary'!$B$4,"Target elapsed",IF(H44&gt;'Executive Summary'!$B$4,"Upcoming","Active window"))))</x:f>
@@ -5619,7 +5582,7 @@
         <x:v>P0</x:v>
       </x:c>
       <x:c r="G45" s="13" t="str">
-        <x:v>To Do</x:v>
+        <x:v>In Progress</x:v>
       </x:c>
       <x:c r="H45" s="191" t="n">
         <x:v>46316</x:v>
@@ -5656,7 +5619,7 @@
 GitHub open/-</x:v>
       </x:c>
       <x:c r="R45" s="13" t="str">
-        <x:v>https://github.com/321Team/fds-project-baseline/issues/47</x:v>
+        <x:v>https://github.com/321Team/fds-project-baseline/issues/47 · 조회 2026-10-19T19:25 KST · body SHA c7b87656feb9</x:v>
       </x:c>
       <x:c r="S45" s="13" t="str">
         <x:f>IF(G45="Done","Done",IF(I45="","End TBD",IF(I45&lt;'Executive Summary'!$B$4,"Target elapsed",IF(H45&gt;'Executive Summary'!$B$4,"Upcoming","Active window"))))</x:f>
@@ -5709,12 +5672,10 @@
         <x:v>D23이 Hybrid DNS를 선택한 경우 Resolver/Conditional Forwarding/Route/Query Test PASS; IP Endpoint 유지 시 Cancelled 결정 근거 승인</x:v>
       </x:c>
       <x:c r="Q46" s="195" t="str">
-        <x:v>P1 Conditional. D23가 Hybrid DNS Go이고 P0 일정 여유가 있을 때만 실행한다. 그렇지 않으면 Cancelled/Deferred 근거를 남기고 IP Endpoint로 P0 E2E를 진행한다.
-GitHub open/-
-원문 일정: TBD — D23 Go + P0 잔여 capacity 시 / TBD — 10-26 이전 강제하지 않음</x:v>
+        <x:v>보류(Deferred) — 2026-10-14 이권욱 결정. 추가 Hybrid DNS 구현을 보류하며 OPEN 유지; Cancelled/완료 아님. Owner 이권욱. D23 Go와 P0 잔여 capacity 및 이권욱의 별도 재개 판단 전 구현하지 않는다. 기존 계획 기준: P1 Conditional. D23가 Hybrid DNS Go이고 P0 일정 여유가 있을 때만 실행한다. 그렇지 않으면 Cancelled/Deferred 근거를 남기고 IP Endpoint로 P0 E2E를 진행한다.</x:v>
       </x:c>
       <x:c r="R46" s="13" t="str">
-        <x:v>https://github.com/321Team/fds-project-baseline/issues/48</x:v>
+        <x:v>https://github.com/321Team/fds-project-baseline/issues/48 · 조회 2026-10-19T19:25 KST · body SHA 15ae082d9a00</x:v>
       </x:c>
       <x:c r="S46" s="13" t="str">
         <x:f>IF(G46="Done","Done",IF(I46="","End TBD",IF(I46&lt;'Executive Summary'!$B$4,"Target elapsed",IF(H46&gt;'Executive Summary'!$B$4,"Upcoming","Active window"))))</x:f>
@@ -5741,7 +5702,7 @@
         <x:v>P0</x:v>
       </x:c>
       <x:c r="G47" s="13" t="str">
-        <x:v>To Do</x:v>
+        <x:v>In Progress</x:v>
       </x:c>
       <x:c r="H47" s="191" t="n">
         <x:v>46318</x:v>
@@ -5778,7 +5739,7 @@
 GitHub open/-</x:v>
       </x:c>
       <x:c r="R47" s="13" t="str">
-        <x:v>https://github.com/321Team/fds-project-baseline/issues/49</x:v>
+        <x:v>https://github.com/321Team/fds-project-baseline/issues/49 · 조회 2026-10-19T19:25 KST · body SHA 0df84e2a05a4</x:v>
       </x:c>
       <x:c r="S47" s="13" t="str">
         <x:f>IF(G47="Done","Done",IF(I47="","End TBD",IF(I47&lt;'Executive Summary'!$B$4,"Target elapsed",IF(H47&gt;'Executive Summary'!$B$4,"Upcoming","Active window"))))</x:f>
@@ -5842,7 +5803,7 @@
 GitHub open/-</x:v>
       </x:c>
       <x:c r="R48" s="13" t="str">
-        <x:v>https://github.com/321Team/fds-project-baseline/issues/50</x:v>
+        <x:v>https://github.com/321Team/fds-project-baseline/issues/50 · 조회 2026-10-19T19:25 KST · body SHA ce799b772f77</x:v>
       </x:c>
       <x:c r="S48" s="13" t="str">
         <x:f>IF(G48="Done","Done",IF(I48="","End TBD",IF(I48&lt;'Executive Summary'!$B$4,"Target elapsed",IF(H48&gt;'Executive Summary'!$B$4,"Upcoming","Active window"))))</x:f>
@@ -5900,7 +5861,7 @@
 원문 일정: TBD — D26 Mirror + P0 잔여 capacity 시 / TBD — 10-26 이전 강제하지 않음</x:v>
       </x:c>
       <x:c r="R49" s="13" t="str">
-        <x:v>https://github.com/321Team/fds-project-baseline/issues/51</x:v>
+        <x:v>https://github.com/321Team/fds-project-baseline/issues/51 · 조회 2026-10-19T19:25 KST · body SHA de786af55724</x:v>
       </x:c>
       <x:c r="S49" s="13" t="str">
         <x:f>IF(G49="Done","Done",IF(I49="","End TBD",IF(I49&lt;'Executive Summary'!$B$4,"Target elapsed",IF(H49&gt;'Executive Summary'!$B$4,"Upcoming","Active window"))))</x:f>
@@ -5927,7 +5888,7 @@
         <x:v>P0</x:v>
       </x:c>
       <x:c r="G50" s="13" t="str">
-        <x:v>To Do</x:v>
+        <x:v>In Progress</x:v>
       </x:c>
       <x:c r="H50" s="191" t="n">
         <x:v>46302</x:v>
@@ -5963,11 +5924,11 @@
 GitHub open/-</x:v>
       </x:c>
       <x:c r="R50" s="13" t="str">
-        <x:v>https://github.com/321Team/fds-project-baseline/issues/52</x:v>
+        <x:v>https://github.com/321Team/fds-project-baseline/issues/52 · 조회 2026-10-19T19:25 KST · body SHA 0bfffefa3778</x:v>
       </x:c>
       <x:c r="S50" s="13" t="str">
         <x:f>IF(G50="Done","Done",IF(I50="","End TBD",IF(I50&lt;'Executive Summary'!$B$4,"Target elapsed",IF(H50&gt;'Executive Summary'!$B$4,"Upcoming","Active window"))))</x:f>
-        <x:v>Upcoming</x:v>
+        <x:v>Target elapsed</x:v>
       </x:c>
     </x:row>
     <x:row r="51" ht="110" customHeight="1">
@@ -6026,7 +5987,7 @@
 GitHub open/-</x:v>
       </x:c>
       <x:c r="R51" s="13" t="str">
-        <x:v>https://github.com/321Team/fds-project-baseline/issues/53</x:v>
+        <x:v>https://github.com/321Team/fds-project-baseline/issues/53 · 조회 2026-10-19T19:25 KST · body SHA bd76c074cec2</x:v>
       </x:c>
       <x:c r="S51" s="13" t="str">
         <x:f>IF(G51="Done","Done",IF(I51="","End TBD",IF(I51&lt;'Executive Summary'!$B$4,"Target elapsed",IF(H51&gt;'Executive Summary'!$B$4,"Upcoming","Active window"))))</x:f>
@@ -6089,7 +6050,7 @@
 GitHub open/-</x:v>
       </x:c>
       <x:c r="R52" s="13" t="str">
-        <x:v>https://github.com/321Team/fds-project-baseline/issues/54</x:v>
+        <x:v>https://github.com/321Team/fds-project-baseline/issues/54 · 조회 2026-10-19T19:25 KST · body SHA 6feb7b1fdc14</x:v>
       </x:c>
       <x:c r="S52" s="13" t="str">
         <x:f>IF(G52="Done","Done",IF(I52="","End TBD",IF(I52&lt;'Executive Summary'!$B$4,"Target elapsed",IF(H52&gt;'Executive Summary'!$B$4,"Upcoming","Active window"))))</x:f>
@@ -6116,7 +6077,7 @@
         <x:v>P0</x:v>
       </x:c>
       <x:c r="G53" s="13" t="str">
-        <x:v>To Do</x:v>
+        <x:v>In Progress</x:v>
       </x:c>
       <x:c r="H53" s="191" t="n">
         <x:v>46318</x:v>
@@ -6152,7 +6113,7 @@
 GitHub open/-</x:v>
       </x:c>
       <x:c r="R53" s="13" t="str">
-        <x:v>https://github.com/321Team/fds-project-baseline/issues/55</x:v>
+        <x:v>https://github.com/321Team/fds-project-baseline/issues/55 · 조회 2026-10-19T19:25 KST · body SHA 855e8842396a</x:v>
       </x:c>
       <x:c r="S53" s="13" t="str">
         <x:f>IF(G53="Done","Done",IF(I53="","End TBD",IF(I53&lt;'Executive Summary'!$B$4,"Target elapsed",IF(H53&gt;'Executive Summary'!$B$4,"Upcoming","Active window"))))</x:f>
@@ -6215,7 +6176,7 @@
 GitHub open/-</x:v>
       </x:c>
       <x:c r="R54" s="13" t="str">
-        <x:v>https://github.com/321Team/fds-project-baseline/issues/56</x:v>
+        <x:v>https://github.com/321Team/fds-project-baseline/issues/56 · 조회 2026-10-19T19:25 KST · body SHA f799554206c2</x:v>
       </x:c>
       <x:c r="S54" s="13" t="str">
         <x:f>IF(G54="Done","Done",IF(I54="","End TBD",IF(I54&lt;'Executive Summary'!$B$4,"Target elapsed",IF(H54&gt;'Executive Summary'!$B$4,"Upcoming","Active window"))))</x:f>
@@ -6278,7 +6239,7 @@
 GitHub open/-</x:v>
       </x:c>
       <x:c r="R55" s="83" t="str">
-        <x:v>https://github.com/321Team/fds-project-baseline/issues/57</x:v>
+        <x:v>https://github.com/321Team/fds-project-baseline/issues/57 · 조회 2026-10-19T19:25 KST · body SHA 0f90761d5ed3</x:v>
       </x:c>
       <x:c r="S55" s="83" t="str">
         <x:f>IF(G55="Done","Done",IF(I55="","End TBD",IF(I55&lt;'Executive Summary'!$B$4,"Target elapsed",IF(H55&gt;'Executive Summary'!$B$4,"Upcoming","Active window"))))</x:f>
@@ -6341,7 +6302,7 @@
 GitHub closed/completed</x:v>
       </x:c>
       <x:c r="R56" s="83" t="str">
-        <x:v>https://github.com/321Team/fds-project-baseline/issues/4</x:v>
+        <x:v>https://github.com/321Team/fds-project-baseline/issues/4 · 조회 2026-10-19T19:25 KST · body SHA 46c9744cb01d · 실제종결 2026-09-09T15:37:02+09:00 (completed)</x:v>
       </x:c>
       <x:c r="S56" s="83" t="str">
         <x:f>IF(G56="Done","Done",IF(I56="","End TBD",IF(I56&lt;'Executive Summary'!$B$4,"Target elapsed",IF(H56&gt;'Executive Summary'!$B$4,"Upcoming","Active window"))))</x:f>
@@ -6404,7 +6365,7 @@
 GitHub closed/completed</x:v>
       </x:c>
       <x:c r="R57" s="83" t="str">
-        <x:v>https://github.com/321Team/fds-project-baseline/issues/5</x:v>
+        <x:v>https://github.com/321Team/fds-project-baseline/issues/5 · 조회 2026-10-19T19:25 KST · body SHA ebf035d43ba3 · 실제종결 2026-09-09T15:37:13+09:00 (completed)</x:v>
       </x:c>
       <x:c r="S57" s="83" t="str">
         <x:f>IF(G57="Done","Done",IF(I57="","End TBD",IF(I57&lt;'Executive Summary'!$B$4,"Target elapsed",IF(H57&gt;'Executive Summary'!$B$4,"Upcoming","Active window"))))</x:f>
@@ -6467,7 +6428,7 @@
 GitHub closed/completed</x:v>
       </x:c>
       <x:c r="R58" s="83" t="str">
-        <x:v>https://github.com/321Team/fds-project-baseline/issues/6</x:v>
+        <x:v>https://github.com/321Team/fds-project-baseline/issues/6 · 조회 2026-10-19T19:25 KST · body SHA bbf7b122c229 · 실제종결 2026-09-09T15:37:24+09:00 (completed)</x:v>
       </x:c>
       <x:c r="S58" s="83" t="str">
         <x:f>IF(G58="Done","Done",IF(I58="","End TBD",IF(I58&lt;'Executive Summary'!$B$4,"Target elapsed",IF(H58&gt;'Executive Summary'!$B$4,"Upcoming","Active window"))))</x:f>
@@ -6530,7 +6491,7 @@
 GitHub closed/completed</x:v>
       </x:c>
       <x:c r="R59" s="148" t="str">
-        <x:v>https://github.com/321Team/fds-project-baseline/issues/74</x:v>
+        <x:v>https://github.com/321Team/fds-project-baseline/issues/74 · 조회 2026-10-19T19:25 KST · body SHA 8032fb1c24b4 · 실제종결 2026-09-26T11:29:06+09:00 (completed)</x:v>
       </x:c>
       <x:c r="S59" s="148" t="str">
         <x:f>IF(G59="Done","Done",IF(I59="","End TBD",IF(I59&lt;'Executive Summary'!$B$4,"Target elapsed",IF(H59&gt;'Executive Summary'!$B$4,"Upcoming","Active window"))))</x:f>
@@ -6593,7 +6554,7 @@
 GitHub closed/completed</x:v>
       </x:c>
       <x:c r="R60" s="148" t="str">
-        <x:v>https://github.com/321Team/fds-project-baseline/issues/75</x:v>
+        <x:v>https://github.com/321Team/fds-project-baseline/issues/75 · 조회 2026-10-19T19:25 KST · body SHA 5e48969d31bc · 실제종결 2026-09-26T19:51:24+09:00 (completed)</x:v>
       </x:c>
       <x:c r="S60" s="148" t="str">
         <x:f>IF(G60="Done","Done",IF(I60="","End TBD",IF(I60&lt;'Executive Summary'!$B$4,"Target elapsed",IF(H60&gt;'Executive Summary'!$B$4,"Upcoming","Active window"))))</x:f>
@@ -6656,7 +6617,7 @@
 GitHub closed/completed</x:v>
       </x:c>
       <x:c r="R61" s="148" t="str">
-        <x:v>https://github.com/321Team/fds-project-baseline/issues/78</x:v>
+        <x:v>https://github.com/321Team/fds-project-baseline/issues/78 · 조회 2026-10-19T19:25 KST · body SHA 3f09efe53d1f · 실제종결 2026-09-16T18:59:17+09:00 (completed)</x:v>
       </x:c>
       <x:c r="S61" s="148" t="str">
         <x:f>IF(G61="Done","Done",IF(I61="","End TBD",IF(I61&lt;'Executive Summary'!$B$4,"Target elapsed",IF(H61&gt;'Executive Summary'!$B$4,"Upcoming","Active window"))))</x:f>
@@ -6719,7 +6680,7 @@
 GitHub closed/completed</x:v>
       </x:c>
       <x:c r="R62" t="str">
-        <x:v>https://github.com/321Team/fds-project-baseline/issues/59</x:v>
+        <x:v>https://github.com/321Team/fds-project-baseline/issues/59 · 조회 2026-10-19T19:25 KST · body SHA c5bc3af88a9d · 실제종결 2026-09-09T18:53:09+09:00 (completed)</x:v>
       </x:c>
       <x:c r="S62" t="str">
         <x:f>IF(G62="Done","Done",IF(I62="","End TBD",IF(I62&lt;'Executive Summary'!$B$4,"Target elapsed",IF(H62&gt;'Executive Summary'!$B$4,"Upcoming","Active window"))))</x:f>
@@ -6782,7 +6743,7 @@
 GitHub closed/completed</x:v>
       </x:c>
       <x:c r="R63" t="str">
-        <x:v>https://github.com/321Team/fds-project-baseline/issues/60</x:v>
+        <x:v>https://github.com/321Team/fds-project-baseline/issues/60 · 조회 2026-10-19T19:25 KST · body SHA ea2f55c13ab4 · 실제종결 2026-09-09T18:53:40+09:00 (completed)</x:v>
       </x:c>
       <x:c r="S63" t="str">
         <x:f>IF(G63="Done","Done",IF(I63="","End TBD",IF(I63&lt;'Executive Summary'!$B$4,"Target elapsed",IF(H63&gt;'Executive Summary'!$B$4,"Upcoming","Active window"))))</x:f>
@@ -6845,7 +6806,7 @@
 GitHub closed/completed</x:v>
       </x:c>
       <x:c r="R64" t="str">
-        <x:v>https://github.com/321Team/fds-project-baseline/issues/61</x:v>
+        <x:v>https://github.com/321Team/fds-project-baseline/issues/61 · 조회 2026-10-19T19:25 KST · body SHA 5f950130e0e4 · 실제종결 2026-09-09T18:54:09+09:00 (completed)</x:v>
       </x:c>
       <x:c r="S64" t="str">
         <x:f>IF(G64="Done","Done",IF(I64="","End TBD",IF(I64&lt;'Executive Summary'!$B$4,"Target elapsed",IF(H64&gt;'Executive Summary'!$B$4,"Upcoming","Active window"))))</x:f>
@@ -6908,7 +6869,7 @@
 GitHub closed/completed</x:v>
       </x:c>
       <x:c r="R65" t="str">
-        <x:v>https://github.com/321Team/fds-project-baseline/issues/62</x:v>
+        <x:v>https://github.com/321Team/fds-project-baseline/issues/62 · 조회 2026-10-19T19:25 KST · body SHA e8cd2a9b4633 · 실제종결 2026-09-09T18:54:41+09:00 (completed)</x:v>
       </x:c>
       <x:c r="S65" t="str">
         <x:f>IF(G65="Done","Done",IF(I65="","End TBD",IF(I65&lt;'Executive Summary'!$B$4,"Target elapsed",IF(H65&gt;'Executive Summary'!$B$4,"Upcoming","Active window"))))</x:f>
@@ -6971,7 +6932,7 @@
 GitHub closed/completed</x:v>
       </x:c>
       <x:c r="R66" t="str">
-        <x:v>https://github.com/321Team/fds-project-baseline/issues/63</x:v>
+        <x:v>https://github.com/321Team/fds-project-baseline/issues/63 · 조회 2026-10-19T19:25 KST · body SHA 61ab60f5943c · 실제종결 2026-09-09T18:55:13+09:00 (completed)</x:v>
       </x:c>
       <x:c r="S66" t="str">
         <x:f>IF(G66="Done","Done",IF(I66="","End TBD",IF(I66&lt;'Executive Summary'!$B$4,"Target elapsed",IF(H66&gt;'Executive Summary'!$B$4,"Upcoming","Active window"))))</x:f>
@@ -7034,7 +6995,7 @@
 GitHub closed/completed</x:v>
       </x:c>
       <x:c r="R67" t="str">
-        <x:v>https://github.com/321Team/fds-project-baseline/issues/64</x:v>
+        <x:v>https://github.com/321Team/fds-project-baseline/issues/64 · 조회 2026-10-19T19:25 KST · body SHA 6d924b398a84 · 실제종결 2026-09-09T18:55:52+09:00 (completed)</x:v>
       </x:c>
       <x:c r="S67" t="str">
         <x:f>IF(G67="Done","Done",IF(I67="","End TBD",IF(I67&lt;'Executive Summary'!$B$4,"Target elapsed",IF(H67&gt;'Executive Summary'!$B$4,"Upcoming","Active window"))))</x:f>
@@ -7097,7 +7058,7 @@
 GitHub closed/completed</x:v>
       </x:c>
       <x:c r="R68" t="str">
-        <x:v>https://github.com/321Team/fds-project-baseline/issues/65</x:v>
+        <x:v>https://github.com/321Team/fds-project-baseline/issues/65 · 조회 2026-10-19T19:25 KST · body SHA fbd2014c6a5b · 실제종결 2026-09-09T18:56:22+09:00 (completed)</x:v>
       </x:c>
       <x:c r="S68" t="str">
         <x:f>IF(G68="Done","Done",IF(I68="","End TBD",IF(I68&lt;'Executive Summary'!$B$4,"Target elapsed",IF(H68&gt;'Executive Summary'!$B$4,"Upcoming","Active window"))))</x:f>
@@ -7160,7 +7121,7 @@
 GitHub closed/completed</x:v>
       </x:c>
       <x:c r="R69" t="str">
-        <x:v>https://github.com/321Team/fds-project-baseline/issues/66</x:v>
+        <x:v>https://github.com/321Team/fds-project-baseline/issues/66 · 조회 2026-10-19T19:25 KST · body SHA 1625eba7ec3e · 실제종결 2026-09-09T18:56:50+09:00 (completed)</x:v>
       </x:c>
       <x:c r="S69" t="str">
         <x:f>IF(G69="Done","Done",IF(I69="","End TBD",IF(I69&lt;'Executive Summary'!$B$4,"Target elapsed",IF(H69&gt;'Executive Summary'!$B$4,"Upcoming","Active window"))))</x:f>
@@ -7223,7 +7184,7 @@
 GitHub closed/completed</x:v>
       </x:c>
       <x:c r="R70" t="str">
-        <x:v>https://github.com/321Team/fds-project-baseline/issues/67</x:v>
+        <x:v>https://github.com/321Team/fds-project-baseline/issues/67 · 조회 2026-10-19T19:25 KST · body SHA f9af2a1aa0b4 · 실제종결 2026-09-09T18:57:19+09:00 (completed)</x:v>
       </x:c>
       <x:c r="S70" t="str">
         <x:f>IF(G70="Done","Done",IF(I70="","End TBD",IF(I70&lt;'Executive Summary'!$B$4,"Target elapsed",IF(H70&gt;'Executive Summary'!$B$4,"Upcoming","Active window"))))</x:f>
@@ -7281,7 +7242,7 @@
 원문 일정: TBD — Deferred 우선 / TBD — 프로젝트 종료 후 별도 PoC는 Project Scope 밖</x:v>
       </x:c>
       <x:c r="R71" t="str">
-        <x:v>https://github.com/321Team/fds-project-baseline/issues/95</x:v>
+        <x:v>https://github.com/321Team/fds-project-baseline/issues/95 · 조회 2026-10-19T19:25 KST · body SHA af713f524931</x:v>
       </x:c>
       <x:c r="S71" t="str">
         <x:f>IF(G71="Done","Done",IF(I71="","End TBD",IF(I71&lt;'Executive Summary'!$B$4,"Target elapsed",IF(H71&gt;'Executive Summary'!$B$4,"Upcoming","Active window"))))</x:f>
@@ -7344,7 +7305,7 @@
 GitHub closed/completed</x:v>
       </x:c>
       <x:c r="R72" t="str">
-        <x:v>https://github.com/321Team/fds-project-baseline/issues/109</x:v>
+        <x:v>https://github.com/321Team/fds-project-baseline/issues/109 · 조회 2026-10-19T19:25 KST · body SHA 446bd362c4cc · 실제종결 2026-09-26T19:51:17+09:00 (completed)</x:v>
       </x:c>
       <x:c r="S72" t="str">
         <x:f>IF(G72="Done","Done",IF(I72="","End TBD",IF(I72&lt;'Executive Summary'!$B$4,"Target elapsed",IF(H72&gt;'Executive Summary'!$B$4,"Upcoming","Active window"))))</x:f>
@@ -7408,7 +7369,7 @@
 GitHub closed/completed</x:v>
       </x:c>
       <x:c r="R73" t="str">
-        <x:v>https://github.com/321Team/fds-project-baseline/issues/110</x:v>
+        <x:v>https://github.com/321Team/fds-project-baseline/issues/110 · 조회 2026-10-19T19:25 KST · body SHA 4b4697034576 · 실제종결 2026-09-27T23:20:19+09:00 (completed)</x:v>
       </x:c>
       <x:c r="S73" t="str">
         <x:f>IF(G73="Done","Done",IF(I73="","End TBD",IF(I73&lt;'Executive Summary'!$B$4,"Target elapsed",IF(H73&gt;'Executive Summary'!$B$4,"Upcoming","Active window"))))</x:f>
@@ -7472,7 +7433,7 @@
 GitHub closed/completed</x:v>
       </x:c>
       <x:c r="R74" t="str">
-        <x:v>https://github.com/321Team/fds-project-baseline/issues/119</x:v>
+        <x:v>https://github.com/321Team/fds-project-baseline/issues/119 · 조회 2026-10-19T19:25 KST · body SHA a7fa8c646d0b · 실제종결 2026-10-01T21:11:06+09:00 (completed)</x:v>
       </x:c>
       <x:c r="S74" t="str">
         <x:f>IF(G74="Done","Done",IF(I74="","End TBD",IF(I74&lt;'Executive Summary'!$B$4,"Target elapsed",IF(H74&gt;'Executive Summary'!$B$4,"Upcoming","Active window"))))</x:f>
@@ -7525,12 +7486,10 @@
         <x:v>OpenShift GitOps 도입/미도입/유예를 단일안으로 결정하고, 도입 시 #46 Delivery Contract 변경 CR·권한모델·Git Source·재생성/Rollback·D26 Operator 공급경로를 승인</x:v>
       </x:c>
       <x:c r="Q75" s="198" t="str">
-        <x:v>P1/non-blocking. #42/#46 P0 Registry/Delivery와 겹치지 않도록 G5 이후 capacity가 있을 때만 Go/No-Go를 판단한다. Go 전에는 기존 Runner direct ROSA Delivery Contract를 유지한다.
-GitHub open/-
-원문 일정: TBD — G5 이후 P0 잔여 capacity 시 / TBD — 10-26 이전 강제하지 않음</x:v>
+        <x:v>보류(Deferred) — 2026-10-14 이권욱 결정. GitOps 도입 결정·구현을 보류하며 기존 Runner direct ROSA Delivery Contract 유지. Owner 이권욱. G5 이후 P0 잔여 capacity와 별도 재개 판단 시에만 재검토; 10/26 이전 착수·완료를 강제하지 않는다. 기존 계획 기준: P1/non-blocking. #42/#46 P0 Registry/Delivery와 겹치지 않도록 G5 이후 capacity가 있을 때만 Go/No-Go를 판단한다. Go 전에는 기존 Runner direct ROSA Delivery Contract를 유지한다.</x:v>
       </x:c>
       <x:c r="R75" t="str">
-        <x:v>https://github.com/321Team/fds-project-baseline/issues/120</x:v>
+        <x:v>https://github.com/321Team/fds-project-baseline/issues/120 · 조회 2026-10-19T19:25 KST · body SHA f623c98cb566</x:v>
       </x:c>
       <x:c r="S75" t="str">
         <x:f>IF(G75="Done","Done",IF(I75="","End TBD",IF(I75&lt;'Executive Summary'!$B$4,"Target elapsed",IF(H75&gt;'Executive Summary'!$B$4,"Upcoming","Active window"))))</x:f>
@@ -7588,7 +7547,7 @@
 원문 일정: TBD — G5 이후 P0 잔여 capacity 시 / TBD — 10-26 이전 강제하지 않음</x:v>
       </x:c>
       <x:c r="R76" t="str">
-        <x:v>https://github.com/321Team/fds-project-baseline/issues/121</x:v>
+        <x:v>https://github.com/321Team/fds-project-baseline/issues/121 · 조회 2026-10-19T19:25 KST · body SHA c709fd2b10dd</x:v>
       </x:c>
       <x:c r="S76" t="str">
         <x:f>IF(G76="Done","Done",IF(I76="","End TBD",IF(I76&lt;'Executive Summary'!$B$4,"Target elapsed",IF(H76&gt;'Executive Summary'!$B$4,"Upcoming","Active window"))))</x:f>
@@ -7652,7 +7611,7 @@
 GitHub closed/completed</x:v>
       </x:c>
       <x:c r="R77" t="str">
-        <x:v>https://github.com/321Team/fds-project-baseline/issues/125</x:v>
+        <x:v>https://github.com/321Team/fds-project-baseline/issues/125 · 조회 2026-10-19T19:25 KST · body SHA 9c54cbf64586 · 실제종결 2026-10-02T12:11:23+09:00 (completed)</x:v>
       </x:c>
       <x:c r="S77" t="str">
         <x:f>IF(G77="Done","Done",IF(I77="","End TBD",IF(I77&lt;'Executive Summary'!$B$4,"Target elapsed",IF(H77&gt;'Executive Summary'!$B$4,"Upcoming","Active window"))))</x:f>
@@ -7679,7 +7638,7 @@
         <x:v>P1</x:v>
       </x:c>
       <x:c r="G78" t="str">
-        <x:v>Done</x:v>
+        <x:v>Cancelled</x:v>
       </x:c>
       <x:c r="H78" s="194" t="n">
         <x:v>46295</x:v>
@@ -7716,11 +7675,11 @@
 GitHub closed/not_planned</x:v>
       </x:c>
       <x:c r="R78" t="str">
-        <x:v>https://github.com/321Team/fds-project-baseline/issues/126</x:v>
+        <x:v>https://github.com/321Team/fds-project-baseline/issues/126 · 조회 2026-10-19T19:25 KST · body SHA 9dd15bd6c419 · 실제종결 2026-10-02T10:30:26+09:00 (not_planned)</x:v>
       </x:c>
       <x:c r="S78" t="str">
         <x:f>IF(G78="Done","Done",IF(I78="","End TBD",IF(I78&lt;'Executive Summary'!$B$4,"Target elapsed",IF(H78&gt;'Executive Summary'!$B$4,"Upcoming","Active window"))))</x:f>
-        <x:v>Done</x:v>
+        <x:v>Target elapsed</x:v>
       </x:c>
     </x:row>
     <x:row r="79" ht="110" customHeight="1">
@@ -7743,7 +7702,7 @@
         <x:v>P1</x:v>
       </x:c>
       <x:c r="G79" t="str">
-        <x:v>Done</x:v>
+        <x:v>Cancelled</x:v>
       </x:c>
       <x:c r="H79" s="194" t="n">
         <x:v>46295</x:v>
@@ -7780,11 +7739,11 @@
 GitHub closed/not_planned</x:v>
       </x:c>
       <x:c r="R79" t="str">
-        <x:v>https://github.com/321Team/fds-project-baseline/issues/127</x:v>
+        <x:v>https://github.com/321Team/fds-project-baseline/issues/127 · 조회 2026-10-19T19:25 KST · body SHA 9fc5e2163bea · 실제종결 2026-10-02T10:34:19+09:00 (not_planned)</x:v>
       </x:c>
       <x:c r="S79" t="str">
         <x:f>IF(G79="Done","Done",IF(I79="","End TBD",IF(I79&lt;'Executive Summary'!$B$4,"Target elapsed",IF(H79&gt;'Executive Summary'!$B$4,"Upcoming","Active window"))))</x:f>
-        <x:v>Done</x:v>
+        <x:v>Target elapsed</x:v>
       </x:c>
     </x:row>
     <x:row r="80" ht="110" customHeight="1">
@@ -7807,7 +7766,7 @@
         <x:v>P1</x:v>
       </x:c>
       <x:c r="G80" t="str">
-        <x:v>Todo</x:v>
+        <x:v>Cancelled</x:v>
       </x:c>
       <x:c r="H80" s="194" t="n">
         <x:v>46295</x:v>
@@ -7827,24 +7786,22 @@
         <x:v>이하영</x:v>
       </x:c>
       <x:c r="M80" t="str">
-        <x:v>미기재</x:v>
+        <x:v>이권욱</x:v>
       </x:c>
       <x:c r="N80" t="str">
         <x:v>D34</x:v>
       </x:c>
       <x:c r="O80" t="str">
-        <x:v>미기재</x:v>
+        <x:v>R1; R2 (본 티켓의 복구·MTU 위험 식별자; 후속 판정은 #10에서 추적)</x:v>
       </x:c>
       <x:c r="P80" s="198" t="str">
         <x:v>#10 핵심 요구 문구 조정 결정 기록(복구 AC 문구는 변경 없음)과 Review Owner 확인, 복구 T19: #10 AC/Exit에 유지하고 worker01 대표 1대 시험 증적(성공 시 복구 AC 수용 근거, 미실행이면 NOT MET / Known Issue), MTU 경로 시험 인정 여부 기록, #125와 통합한 Change Matrix, #10 본문 교체, 차기 정본 Ticket Pack 동기화</x:v>
       </x:c>
       <x:c r="Q80" s="198" t="str">
-        <x:v>원문 Schedule Note 미기재
-WITHDRAWN_NO_AC_CHANGE; body Todo / closed not_planned 차이 보존.
-GitHub closed/not_planned</x:v>
+        <x:v>기존 계획 2026-09-30~2026-10-02(양끝 포함 3일/3근무일) 유지. 2026-10-02 WITHDRAWN / NO AC CHANGE로 종결. Support 이권욱은 기존 Review Owner 및 #10 Support 역할의 운영 표기이며 신규 실행 책임 배정이 아니다. T19 실행 일정·AC는 #10에서 별도 추적.</x:v>
       </x:c>
       <x:c r="R80" t="str">
-        <x:v>https://github.com/321Team/fds-project-baseline/issues/128</x:v>
+        <x:v>https://github.com/321Team/fds-project-baseline/issues/128 · 조회 2026-10-19T19:25 KST · body SHA 5d0558b81e86 · 실제종결 2026-10-02T09:58:57+09:00 (not_planned)</x:v>
       </x:c>
       <x:c r="S80" t="str">
         <x:f>IF(G80="Done","Done",IF(I80="","End TBD",IF(I80&lt;'Executive Summary'!$B$4,"Target elapsed",IF(H80&gt;'Executive Summary'!$B$4,"Upcoming","Active window"))))</x:f>
@@ -7891,24 +7848,22 @@
         <x:v>이하영</x:v>
       </x:c>
       <x:c r="M81" t="str">
-        <x:v>이권욱 (#16 Lead — AC-05B 인수 구조 확인)</x:v>
+        <x:v>이권욱</x:v>
       </x:c>
       <x:c r="N81" t="str">
         <x:v>D19; D-SEC-01; [2026-09-14 Robot 유한 30일 결정](https://github.com/321Team/fds-project-baseline/issues/13#issuecomment-5659049448)</x:v>
       </x:c>
       <x:c r="O81" t="str">
-        <x:v>미기재</x:v>
+        <x:v>별도 CR 위험 ID 미지정; 관련 원 티켓 #13의 RISK-04; RISK-06; RISK-07 참조</x:v>
       </x:c>
       <x:c r="P81" s="198" t="str">
         <x:v>#13 핵심 요구/AC-05 구조 조정 결정 기록, #14의 OID-02 완료조건/Owner/Due 명시, #16 Lead의 4/4 Review Run 산출물 제공 확인, #13 본문 교체</x:v>
       </x:c>
       <x:c r="Q81" s="198" t="str">
-        <x:v>원문 Schedule Note 미기재
-CHG01/02 구조 승인; #16 생산/#13 05B 인수 유지.
-GitHub closed/completed</x:v>
+        <x:v>기존 계획 2026-09-30~2026-10-02(양끝 포함 3일/3근무일) 유지. 실제 CR 완료일은 기존 Completion Record의 2026-10-03이며 계획 End와 구분. Support 이권욱: #16 Lead — AC-05B 인수 구조 확인. Harbor·4/4·Rollback Runtime 일정과 인수는 #13/#16에서 별도 추적.</x:v>
       </x:c>
       <x:c r="R81" t="str">
-        <x:v>https://github.com/321Team/fds-project-baseline/issues/130</x:v>
+        <x:v>https://github.com/321Team/fds-project-baseline/issues/130 · 조회 2026-10-19T19:25 KST · body SHA 60ed458edeef · 실제종결 2026-10-03T11:13:21+09:00 (completed)</x:v>
       </x:c>
       <x:c r="S81" t="str">
         <x:f>IF(G81="Done","Done",IF(I81="","End TBD",IF(I81&lt;'Executive Summary'!$B$4,"Target elapsed",IF(H81&gt;'Executive Summary'!$B$4,"Upcoming","Active window"))))</x:f>
@@ -7959,7 +7914,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5a212b11954840f6"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R941a0259b39a49a6"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -8068,7 +8023,7 @@
     </x:row>
     <x:row r="3">
       <x:c r="A3" t="str">
-        <x:v>Plan windows only. No Runtime completion claim. Current test gates: Test Strategy.</x:v>
+        <x:v>원 Phase1 계획 이력. #25~27 현재 Phase2 이월이며 구현 To Do·Due 미정. 현행 분류는 WBS C열을 따른다.</x:v>
       </x:c>
     </x:row>
     <x:row r="4">
@@ -8248,7 +8203,7 @@
       </x:c>
       <x:c r="C5" s="195" t="str">
         <x:f>WBS!G6</x:f>
-        <x:v>In Progress</x:v>
+        <x:v>Done</x:v>
       </x:c>
       <x:c r="D5" s="225" t="n">
         <x:f>WBS!H6</x:f>
@@ -8597,7 +8552,7 @@
       </x:c>
       <x:c r="C7" s="195" t="str">
         <x:f>WBS!G8</x:f>
-        <x:v>In Progress</x:v>
+        <x:v>Done</x:v>
       </x:c>
       <x:c r="D7" s="225" t="n">
         <x:f>WBS!H8</x:f>
@@ -9610,7 +9565,7 @@
       </x:c>
       <x:c r="C13" s="195" t="str">
         <x:f>WBS!G14</x:f>
-        <x:v>In Progress</x:v>
+        <x:v>Done</x:v>
       </x:c>
       <x:c r="D13" s="225" t="n">
         <x:f>WBS!H14</x:f>
@@ -10450,7 +10405,7 @@
       </x:c>
       <x:c r="C18" s="195" t="str">
         <x:f>WBS!G19</x:f>
-        <x:v>In Progress</x:v>
+        <x:v>Done</x:v>
       </x:c>
       <x:c r="D18" s="225" t="n">
         <x:f>WBS!H19</x:f>
@@ -10619,7 +10574,7 @@
       </x:c>
       <x:c r="C19" s="195" t="str">
         <x:f>WBS!G20</x:f>
-        <x:v>In Progress</x:v>
+        <x:v>Done</x:v>
       </x:c>
       <x:c r="D19" s="225" t="n">
         <x:f>WBS!H20</x:f>
@@ -11925,7 +11880,7 @@
       </x:c>
       <x:c r="C27" s="195" t="str">
         <x:f>WBS!G28</x:f>
-        <x:v>To Do</x:v>
+        <x:v>In Progress</x:v>
       </x:c>
       <x:c r="D27" s="225" t="n">
         <x:f>WBS!H28</x:f>
@@ -12086,7 +12041,7 @@
       </x:c>
       <x:c r="C28" s="195" t="str">
         <x:f>WBS!G29</x:f>
-        <x:v>To Do</x:v>
+        <x:v>In Progress</x:v>
       </x:c>
       <x:c r="D28" s="225" t="n">
         <x:f>WBS!H29</x:f>
@@ -15034,7 +14989,7 @@
       </x:c>
       <x:c r="C46" s="198" t="str">
         <x:f>WBS!G78</x:f>
-        <x:v>Done</x:v>
+        <x:v>Cancelled</x:v>
       </x:c>
       <x:c r="D46" s="226" t="n">
         <x:f>WBS!H78</x:f>
@@ -15197,7 +15152,7 @@
       </x:c>
       <x:c r="C47" s="198" t="str">
         <x:f>WBS!G79</x:f>
-        <x:v>Done</x:v>
+        <x:v>Cancelled</x:v>
       </x:c>
       <x:c r="D47" s="226" t="n">
         <x:f>WBS!H79</x:f>
@@ -15360,7 +15315,7 @@
       </x:c>
       <x:c r="C48" s="198" t="str">
         <x:f>WBS!G80</x:f>
-        <x:v>Todo</x:v>
+        <x:v>Cancelled</x:v>
       </x:c>
       <x:c r="D48" s="226" t="n">
         <x:f>WBS!H80</x:f>
@@ -18225,7 +18180,7 @@
     </x:row>
     <x:row r="3">
       <x:c r="A3" t="str">
-        <x:v>Plan windows only. No Runtime completion claim. Current test gates: Test Strategy.</x:v>
+        <x:v>원 Phase2 계획 창. 이월 #25~27도 현재 Phase2이며 WBS에서 추적. 막대는 Runtime 완료율이 아니다.</x:v>
       </x:c>
     </x:row>
     <x:row r="4">
@@ -18506,7 +18461,7 @@
       </x:c>
       <x:c r="C6" s="195" t="str">
         <x:f>WBS!G32</x:f>
-        <x:v>To Do</x:v>
+        <x:v>Done</x:v>
       </x:c>
       <x:c r="D6" s="225" t="n">
         <x:f>WBS!H32</x:f>
@@ -18637,7 +18592,7 @@
       </x:c>
       <x:c r="C7" s="195" t="str">
         <x:f>WBS!G33</x:f>
-        <x:v>To Do</x:v>
+        <x:v>In Progress</x:v>
       </x:c>
       <x:c r="D7" s="225" t="n">
         <x:f>WBS!H33</x:f>
@@ -18771,7 +18726,7 @@
       </x:c>
       <x:c r="C8" s="195" t="str">
         <x:f>WBS!G34</x:f>
-        <x:v>To Do</x:v>
+        <x:v>In Progress</x:v>
       </x:c>
       <x:c r="D8" s="225" t="n">
         <x:f>WBS!H34</x:f>
@@ -18903,7 +18858,7 @@
       </x:c>
       <x:c r="C9" s="195" t="str">
         <x:f>WBS!G35</x:f>
-        <x:v>To Do</x:v>
+        <x:v>In Progress</x:v>
       </x:c>
       <x:c r="D9" s="225" t="n">
         <x:f>WBS!H35</x:f>
@@ -19036,7 +18991,7 @@
       </x:c>
       <x:c r="C10" s="195" t="str">
         <x:f>WBS!G36</x:f>
-        <x:v>To Do</x:v>
+        <x:v>In Progress</x:v>
       </x:c>
       <x:c r="D10" s="225" t="n">
         <x:f>WBS!H36</x:f>
@@ -19561,7 +19516,7 @@
       </x:c>
       <x:c r="C14" s="195" t="str">
         <x:f>WBS!G40</x:f>
-        <x:v>To Do</x:v>
+        <x:v>In Progress</x:v>
       </x:c>
       <x:c r="D14" s="225" t="n">
         <x:f>WBS!H40</x:f>
@@ -19692,7 +19647,7 @@
       </x:c>
       <x:c r="C15" s="195" t="str">
         <x:f>WBS!G41</x:f>
-        <x:v>To Do</x:v>
+        <x:v>In Progress</x:v>
       </x:c>
       <x:c r="D15" s="225" t="n">
         <x:f>WBS!H41</x:f>
@@ -20085,7 +20040,7 @@
       </x:c>
       <x:c r="C18" s="195" t="str">
         <x:f>WBS!G44</x:f>
-        <x:v>To Do</x:v>
+        <x:v>In Progress</x:v>
       </x:c>
       <x:c r="D18" s="225" t="n">
         <x:f>WBS!H44</x:f>
@@ -20216,7 +20171,7 @@
       </x:c>
       <x:c r="C19" s="195" t="str">
         <x:f>WBS!G45</x:f>
-        <x:v>To Do</x:v>
+        <x:v>In Progress</x:v>
       </x:c>
       <x:c r="D19" s="225" t="n">
         <x:f>WBS!H45</x:f>
@@ -20477,7 +20432,7 @@
       </x:c>
       <x:c r="C21" s="195" t="str">
         <x:f>WBS!G47</x:f>
-        <x:v>To Do</x:v>
+        <x:v>In Progress</x:v>
       </x:c>
       <x:c r="D21" s="225" t="n">
         <x:f>WBS!H47</x:f>
@@ -20869,7 +20824,7 @@
       </x:c>
       <x:c r="C24" s="195" t="str">
         <x:f>WBS!G50</x:f>
-        <x:v>To Do</x:v>
+        <x:v>In Progress</x:v>
       </x:c>
       <x:c r="D24" s="225" t="n">
         <x:f>WBS!H50</x:f>
@@ -21262,7 +21217,7 @@
       </x:c>
       <x:c r="C27" s="195" t="str">
         <x:f>WBS!G53</x:f>
-        <x:v>To Do</x:v>
+        <x:v>In Progress</x:v>
       </x:c>
       <x:c r="D27" s="225" t="n">
         <x:f>WBS!H53</x:f>
@@ -25510,10 +25465,7 @@
       </x:c>
       <x:c r="I6" s="195" t="str">
         <x:f>WBS!Q16</x:f>
-        <x:v>10/19 조건부 인수/판정. 근거 https://github.com/321Team/fds-project-baseline/issues/18#issuecomment-6264597081. 실제 종결 2026-10-19T19:05:40+09:00. 종결 근거 https://github.com/321Team/fds-project-baseline/issues/18#issuecomment-6264709975. 원 AC/계획/Owner와 기술 한계 유지.
-[기존 계획/관측]
-09-17 오후 조건부 인수 목표. 6대·API/LB·Calico·DB·Harbor·Runner 증적 미충족이면 PASS 불가. 실제 상태·완료 판정은 유지한다. 세부 배정: Fast Track Plan 시트.
-GitHub open/-</x:v>
+        <x:v>09-17 오후 조건부 인수 목표. 6대·API/LB·Calico·DB·Harbor·Runner 증적 미충족이면 PASS 불가. 실제 상태·완료 판정은 유지한다. 세부 배정: Fast Track Plan 시트.</x:v>
       </x:c>
       <x:c r="J6" s="195" t="str">
         <x:v>Lifecycle only; Runtime separate</x:v>
@@ -25553,10 +25505,7 @@
       </x:c>
       <x:c r="I7" s="195" t="str">
         <x:f>WBS!Q21</x:f>
-        <x:v>10/19 조건부 인수/판정. 근거 https://github.com/321Team/fds-project-baseline/issues/23#issuecomment-6264221185. 실제 종결 2026-10-19T19:05:48+09:00. 종결 근거 https://github.com/321Team/fds-project-baseline/issues/23#issuecomment-6264712221. 원 AC/계획/Owner와 기술 한계 유지.
-[기존 계획/관측]
-09-21 오후 종료 시점 목표. 앱/보안/CI/Monitoring·초기 E2E/Negative/Drain 준비도와 해당 증적이 선행한다. 실제 상태·완료 판정은 유지한다. 세부 배정: Fast Track Plan 시트.
-GitHub open/-</x:v>
+        <x:v>09-21 오후 종료 시점 목표. 앱/보안/CI/Monitoring·초기 E2E/Negative/Drain 준비도와 해당 증적이 선행한다. 실제 상태·완료 판정은 유지한다. 세부 배정: Fast Track Plan 시트.</x:v>
       </x:c>
       <x:c r="J7" s="195" t="str">
         <x:v>Lifecycle only; Runtime separate</x:v>
@@ -25637,10 +25586,7 @@
       </x:c>
       <x:c r="I9" s="195" t="str">
         <x:f>WBS!Q27</x:f>
-        <x:v>10/19 조건부 인수/판정. 근거 https://github.com/321Team/fds-project-baseline/issues/29#issuecomment-6264597709. 실제 종결 2026-10-19T19:05:55+09:00. 종결 근거 https://github.com/321Team/fds-project-baseline/issues/29#issuecomment-6264714186. 원 AC/계획/Owner와 기술 한계 유지.
-[기존 계획/관측]
-10-02는 실작업·증적 cutoff/G3 Review Ready 판정일이다. 남은 Phase 1 P0는 담당자별 공유 Runtime으로 직렬화하고, 미완료 AC는 10-06 Review에서 사실 상태를 분류한다. 일정 도래만으로 Gate PASS 처리하지 않는다.
-GitHub open/-</x:v>
+        <x:v>10-02는 실작업·증적 cutoff/G3 Review Ready 판정일이다. 남은 Phase 1 P0는 담당자별 공유 Runtime으로 직렬화하고, 미완료 AC는 10-06 Review에서 사실 상태를 분류한다. 일정 도래만으로 Gate PASS 처리하지 않는다.</x:v>
       </x:c>
       <x:c r="J9" s="195" t="str">
         <x:v>Lifecycle only; Runtime separate</x:v>
@@ -25661,7 +25607,7 @@
       </x:c>
       <x:c r="D10" s="13" t="str">
         <x:f>WBS!G29</x:f>
-        <x:v>To Do</x:v>
+        <x:v>In Progress</x:v>
       </x:c>
       <x:c r="E10" s="191" t="n">
         <x:f>WBS!H29</x:f>
@@ -25784,7 +25730,7 @@
       </x:c>
       <x:c r="D13" s="13" t="str">
         <x:f>WBS!G34</x:f>
-        <x:v>To Do</x:v>
+        <x:v>In Progress</x:v>
       </x:c>
       <x:c r="E13" s="191" t="n">
         <x:f>WBS!H34</x:f>
@@ -25886,9 +25832,7 @@
       </x:c>
       <x:c r="I15" s="195" t="str">
         <x:f>WBS!Q38</x:f>
-        <x:v>P0 Hybrid 경로 차단을 피하기 위해 10-16 단일 Decision window에서 IP Endpoint 유지 또는 DNS P1 적용을 확정한다. 구현(#48)은 Go이면서 P0 잔여 capacity가 있을 때만 별도 착수한다.
-TS04; 전체 P1 유지. private 필수 DNS subset은 pre-create 계약.
-GitHub open/-</x:v>
+        <x:v>보류(Deferred) — 2026-10-14 이권욱 결정. D23 추가 Hybrid DNS 도입 보류 확정; 기존 DB/Harbor IP 및 ROSA public API/Route DNS·엄격 TLS 기준 유지. Owner 이권욱. 기존10/16은 보류 재검토 기준일이며 자동 재개 승인이 아니다. 재개는 이권욱의 별도 판단 후 결정. 기존 계획 기준: P0 Hybrid 경로 차단을 피하기 위해 10-16 단일 Decision window에서 IP Endpoint 유지 또는 DNS P1 적용을 확정한다. 구현(#48)은 Go이면서 P0 잔여 capacity가 있을 때만 별도 착수한다.</x:v>
       </x:c>
       <x:c r="J15" s="195" t="str">
         <x:v>TS04; 전체 P1 유지. private 필수 DNS subset은 pre-create 계약.</x:v>
@@ -25951,7 +25895,7 @@
       </x:c>
       <x:c r="D17" s="13" t="str">
         <x:f>WBS!G40</x:f>
-        <x:v>To Do</x:v>
+        <x:v>In Progress</x:v>
       </x:c>
       <x:c r="E17" s="191" t="n">
         <x:f>WBS!H40</x:f>
@@ -26034,7 +25978,7 @@
       </x:c>
       <x:c r="D19" s="67" t="str">
         <x:f>WBS!G50</x:f>
-        <x:v>To Do</x:v>
+        <x:v>In Progress</x:v>
       </x:c>
       <x:c r="E19" s="229" t="n">
         <x:f>WBS!H50</x:f>
@@ -26670,9 +26614,7 @@
       </x:c>
       <x:c r="I34" s="197" t="str">
         <x:f>WBS!Q75</x:f>
-        <x:v>P1/non-blocking. #42/#46 P0 Registry/Delivery와 겹치지 않도록 G5 이후 capacity가 있을 때만 Go/No-Go를 판단한다. Go 전에는 기존 Runner direct ROSA Delivery Contract를 유지한다.
-GitHub open/-
-원문 일정: TBD — G5 이후 P0 잔여 capacity 시 / TBD — 10-26 이전 강제하지 않음</x:v>
+        <x:v>보류(Deferred) — 2026-10-14 이권욱 결정. GitOps 도입 결정·구현을 보류하며 기존 Runner direct ROSA Delivery Contract 유지. Owner 이권욱. G5 이후 P0 잔여 capacity와 별도 재개 판단 시에만 재검토; 10/26 이전 착수·완료를 강제하지 않는다. 기존 계획 기준: P1/non-blocking. #42/#46 P0 Registry/Delivery와 겹치지 않도록 G5 이후 capacity가 있을 때만 Go/No-Go를 판단한다. Go 전에는 기존 Runner direct ROSA Delivery Contract를 유지한다.</x:v>
       </x:c>
       <x:c r="J34" s="197" t="str">
         <x:v>Lifecycle only; Runtime separate</x:v>
@@ -27482,7 +27424,7 @@
         <x:v>2026-10-03</x:v>
       </x:c>
       <x:c r="E4" s="13" t="str">
-        <x:v>78 Issue snapshot; historical rows remain dated.</x:v>
+        <x:v>v3.1.21 원본 보존. 현재78건은 10/19 GitHub 조회와 후속 승인 반영 후보.</x:v>
       </x:c>
       <x:c r="G4" s="13" t="inlineStr">
         <x:is>

</xml_diff>

<commit_message>
docs: record actual bounded Review31 adoption (adopted)
</commit_message>
<xml_diff>
--- a/audit/canonical-candidate-20261019/proposed/FDS_P1_WBS_Status_Candidate_20261019.xlsx
+++ b/audit/canonical-candidate-20261019/proposed/FDS_P1_WBS_Status_Candidate_20261019.xlsx
@@ -2,16 +2,16 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Executive Summary" sheetId="1" r:id="R42f3e076264c4eb7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="WBS" sheetId="2" r:id="R708f3804f8e6408c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase 1 Gantt" sheetId="3" r:id="R4e0843d731ce47b5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase 2 Gantt" sheetId="4" r:id="Ra8c9a790392e4347"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Milestones &amp; Decisions" sheetId="5" r:id="Ra5a5e20e8aa84886"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risks &amp; Assumptions" sheetId="6" r:id="R90958ae79ffe4113"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources &amp; Change Log" sheetId="7" r:id="Rf58d195b06d04aba"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Team Calendar" sheetId="8" r:id="R0d32c6285c854eb5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fast Track Plan" sheetId="9" r:id="Ra558d84348154995"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Strategy" sheetId="10" r:id="R48c9a11a844e4559"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Executive Summary" sheetId="1" r:id="Rf0e2dc9e1d8741f4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="WBS" sheetId="2" r:id="R2f32bb350f6c48fe"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase 1 Gantt" sheetId="3" r:id="R5dc516571d1149ed"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase 2 Gantt" sheetId="4" r:id="R0945211073214ec0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Milestones &amp; Decisions" sheetId="5" r:id="Rb6985db979224d1f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risks &amp; Assumptions" sheetId="6" r:id="R4e39557b1876493b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources &amp; Change Log" sheetId="7" r:id="R68884278a28e45ba"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Team Calendar" sheetId="8" r:id="R41d85fe6096e4258"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fast Track Plan" sheetId="9" r:id="R1fd14f0e2f904ee7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Strategy" sheetId="10" r:id="Rac60ae5522c8437e"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1762,7 +1762,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R1124a92c80e944b1"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R9307a102ebed4382"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1792,7 +1792,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Re4c0e19a97d644de"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R905ef6d5054d4acc"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -2495,7 +2495,7 @@
     <x:mergeCell ref="A18:V18"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdb06801cefe24b79"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5f36b9ebcd524734"/>
 </x:worksheet>
 </file>
 
@@ -4610,7 +4610,7 @@
       </x:c>
       <x:c r="Q29" s="195" t="str">
         <x:v>2026-09-23 Lead 결정으로 09-22에서 10-06(화)으로 조정. 같은 날 #30 보완·Sign-off와 #32 Close로 이어진다. G3 통과와 참석자 확정이 필요하다. 실제 상태·완료 판정은 유지한다.
-GitHub open/-</x:v>
+GitHub open/- · 10/19 사용자 비동기 증적 Review 방식/최종결과 한정 채택. 실제 기록 https://github.com/321Team/fds-project-baseline/issues/31#issuecomment-6265340124 · 관리 결과 반영 후 티켓 종결 예정. #30 Signoff/#32 Close 별도.</x:v>
       </x:c>
       <x:c r="R29" s="13" t="str">
         <x:v>https://github.com/321Team/fds-project-baseline/issues/31 · 조회 2026-10-19T19:25 KST · body SHA 7b0b4bb69e61</x:v>
@@ -7914,7 +7914,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R941a0259b39a49a6"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb71e844e7c6d4bd3"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -25627,7 +25627,7 @@
       <x:c r="I10" s="195" t="str">
         <x:f>WBS!Q29</x:f>
         <x:v>2026-09-23 Lead 결정으로 09-22에서 10-06(화)으로 조정. 같은 날 #30 보완·Sign-off와 #32 Close로 이어진다. G3 통과와 참석자 확정이 필요하다. 실제 상태·완료 판정은 유지한다.
-GitHub open/-</x:v>
+GitHub open/- · 10/19 사용자 비동기 증적 Review 방식/최종결과 한정 채택. 실제 기록 https://github.com/321Team/fds-project-baseline/issues/31#issuecomment-6265340124 · 관리 결과 반영 후 티켓 종결 예정. #30 Signoff/#32 Close 별도.</x:v>
       </x:c>
       <x:c r="J10" s="195" t="str">
         <x:v>Lifecycle only; Runtime separate</x:v>

</xml_diff>

<commit_message>
docs: record actual bounded Review31 adoption (closed)
</commit_message>
<xml_diff>
--- a/audit/canonical-candidate-20261019/proposed/FDS_P1_WBS_Status_Candidate_20261019.xlsx
+++ b/audit/canonical-candidate-20261019/proposed/FDS_P1_WBS_Status_Candidate_20261019.xlsx
@@ -2,16 +2,16 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Executive Summary" sheetId="1" r:id="Rf0e2dc9e1d8741f4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="WBS" sheetId="2" r:id="R2f32bb350f6c48fe"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase 1 Gantt" sheetId="3" r:id="R5dc516571d1149ed"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase 2 Gantt" sheetId="4" r:id="R0945211073214ec0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Milestones &amp; Decisions" sheetId="5" r:id="Rb6985db979224d1f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risks &amp; Assumptions" sheetId="6" r:id="R4e39557b1876493b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources &amp; Change Log" sheetId="7" r:id="R68884278a28e45ba"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Team Calendar" sheetId="8" r:id="R41d85fe6096e4258"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fast Track Plan" sheetId="9" r:id="R1fd14f0e2f904ee7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Strategy" sheetId="10" r:id="Rac60ae5522c8437e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Executive Summary" sheetId="1" r:id="Re9742af802054c0e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="WBS" sheetId="2" r:id="R3dfa9ac6f5154811"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase 1 Gantt" sheetId="3" r:id="R9826e58b1396464a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase 2 Gantt" sheetId="4" r:id="Re8fbbbb693534c60"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Milestones &amp; Decisions" sheetId="5" r:id="R8728a883d9a84d64"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risks &amp; Assumptions" sheetId="6" r:id="Reb3d61ce8c4f4e82"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources &amp; Change Log" sheetId="7" r:id="R813d69e850af455f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Team Calendar" sheetId="8" r:id="Reca0554af1334ead"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fast Track Plan" sheetId="9" r:id="R6602224478724a7e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Strategy" sheetId="10" r:id="R1e07e56eeb3c4a4f"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1762,7 +1762,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R9307a102ebed4382"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rb4f270c219a54f50"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1792,7 +1792,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R905ef6d5054d4acc"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R0afa5321836a4e25"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -2114,7 +2114,7 @@
         <x:v>P1 Close</x:v>
       </x:c>
       <x:c r="E4" s="199" t="str">
-        <x:v>Review 진행 · Signoff 미완료</x:v>
+        <x:v>Review 채택 완료 · Signoff 잔여</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="32" customHeight="1">
@@ -2228,7 +2228,7 @@
       </x:c>
       <x:c r="B12" s="13" t="n">
         <x:f>COUNTIF(WBS!$G$4:$G$81,A12)</x:f>
-        <x:v>42</x:v>
+        <x:v>43</x:v>
       </x:c>
       <x:c r="D12" s="13" t="inlineStr">
         <x:is>
@@ -2248,7 +2248,7 @@
       </x:c>
       <x:c r="B13" s="13" t="n">
         <x:f>COUNTIF(WBS!$G$4:$G$81,A13)</x:f>
-        <x:v>13</x:v>
+        <x:v>12</x:v>
       </x:c>
       <x:c r="D13" s="13" t="inlineStr">
         <x:is>
@@ -2372,7 +2372,7 @@
         <x:v>P1 Close</x:v>
       </x:c>
       <x:c r="C21" s="13" t="str">
-        <x:v>모듈·G1~G3 조건부 인수 완료. #31 Review/#30 Signoff/#32 Close 잔여.</x:v>
+        <x:v>모듈·G1~G3·#31 조건부 Review 인수 완료. #30 Signoff/#32 Close 잔여.</x:v>
       </x:c>
       <x:c r="D21" s="195" t="str">
         <x:v>각 P1 Lead</x:v>
@@ -2495,7 +2495,7 @@
     <x:mergeCell ref="A18:V18"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5f36b9ebcd524734"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd5409e5d48684c00"/>
 </x:worksheet>
 </file>
 
@@ -4577,7 +4577,7 @@
         <x:v>P0</x:v>
       </x:c>
       <x:c r="G29" s="13" t="str">
-        <x:v>In Progress</x:v>
+        <x:v>Done</x:v>
       </x:c>
       <x:c r="H29" s="191" t="n">
         <x:v>46301</x:v>
@@ -4610,14 +4610,14 @@
       </x:c>
       <x:c r="Q29" s="195" t="str">
         <x:v>2026-09-23 Lead 결정으로 09-22에서 10-06(화)으로 조정. 같은 날 #30 보완·Sign-off와 #32 Close로 이어진다. G3 통과와 참석자 확정이 필요하다. 실제 상태·완료 판정은 유지한다.
-GitHub open/- · 10/19 사용자 비동기 증적 Review 방식/최종결과 한정 채택. 실제 기록 https://github.com/321Team/fds-project-baseline/issues/31#issuecomment-6265340124 · 관리 결과 반영 후 티켓 종결 예정. #30 Signoff/#32 Close 별도.</x:v>
+GitHub open/- · 10/19 사용자 비동기 증적 Review 방식/최종결과 한정 채택. 실제 기록 https://github.com/321Team/fds-project-baseline/issues/31#issuecomment-6265340124 · 실제 closed(completed) 2026-10-19T19:45:18+09:00. #30 Signoff/#32 Close 별도.</x:v>
       </x:c>
       <x:c r="R29" s="13" t="str">
-        <x:v>https://github.com/321Team/fds-project-baseline/issues/31 · 조회 2026-10-19T19:25 KST · body SHA 7b0b4bb69e61</x:v>
+        <x:v>https://github.com/321Team/fds-project-baseline/issues/31 · 실제종결 2026-10-19T19:45:18+09:00 · body SHA 74b462cf3f0a · 실제Review채택 https://github.com/321Team/fds-project-baseline/issues/31#issuecomment-6265340124</x:v>
       </x:c>
       <x:c r="S29" s="13" t="str">
         <x:f>IF(G29="Done","Done",IF(I29="","End TBD",IF(I29&lt;'Executive Summary'!$B$4,"Target elapsed",IF(H29&gt;'Executive Summary'!$B$4,"Upcoming","Active window"))))</x:f>
-        <x:v>Target elapsed</x:v>
+        <x:v>Done</x:v>
       </x:c>
     </x:row>
     <x:row r="30" ht="110" customHeight="1">
@@ -7914,7 +7914,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb71e844e7c6d4bd3"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbba67dac05554f84"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -12041,7 +12041,7 @@
       </x:c>
       <x:c r="C28" s="195" t="str">
         <x:f>WBS!G29</x:f>
-        <x:v>In Progress</x:v>
+        <x:v>Done</x:v>
       </x:c>
       <x:c r="D28" s="225" t="n">
         <x:f>WBS!H29</x:f>
@@ -25607,7 +25607,7 @@
       </x:c>
       <x:c r="D10" s="13" t="str">
         <x:f>WBS!G29</x:f>
-        <x:v>In Progress</x:v>
+        <x:v>Done</x:v>
       </x:c>
       <x:c r="E10" s="191" t="n">
         <x:f>WBS!H29</x:f>
@@ -25627,7 +25627,7 @@
       <x:c r="I10" s="195" t="str">
         <x:f>WBS!Q29</x:f>
         <x:v>2026-09-23 Lead 결정으로 09-22에서 10-06(화)으로 조정. 같은 날 #30 보완·Sign-off와 #32 Close로 이어진다. G3 통과와 참석자 확정이 필요하다. 실제 상태·완료 판정은 유지한다.
-GitHub open/- · 10/19 사용자 비동기 증적 Review 방식/최종결과 한정 채택. 실제 기록 https://github.com/321Team/fds-project-baseline/issues/31#issuecomment-6265340124 · 관리 결과 반영 후 티켓 종결 예정. #30 Signoff/#32 Close 별도.</x:v>
+GitHub open/- · 10/19 사용자 비동기 증적 Review 방식/최종결과 한정 채택. 실제 기록 https://github.com/321Team/fds-project-baseline/issues/31#issuecomment-6265340124 · 실제 closed(completed) 2026-10-19T19:45:18+09:00. #30 Signoff/#32 Close 별도.</x:v>
       </x:c>
       <x:c r="J10" s="195" t="str">
         <x:v>Lifecycle only; Runtime separate</x:v>

</xml_diff>

<commit_message>
docs: record actual bounded Review31 adoption (final-note)
</commit_message>
<xml_diff>
--- a/audit/canonical-candidate-20261019/proposed/FDS_P1_WBS_Status_Candidate_20261019.xlsx
+++ b/audit/canonical-candidate-20261019/proposed/FDS_P1_WBS_Status_Candidate_20261019.xlsx
@@ -2,16 +2,16 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Executive Summary" sheetId="1" r:id="Re9742af802054c0e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="WBS" sheetId="2" r:id="R3dfa9ac6f5154811"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase 1 Gantt" sheetId="3" r:id="R9826e58b1396464a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase 2 Gantt" sheetId="4" r:id="Re8fbbbb693534c60"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Milestones &amp; Decisions" sheetId="5" r:id="R8728a883d9a84d64"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risks &amp; Assumptions" sheetId="6" r:id="Reb3d61ce8c4f4e82"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources &amp; Change Log" sheetId="7" r:id="R813d69e850af455f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Team Calendar" sheetId="8" r:id="Reca0554af1334ead"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fast Track Plan" sheetId="9" r:id="R6602224478724a7e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Strategy" sheetId="10" r:id="R1e07e56eeb3c4a4f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Executive Summary" sheetId="1" r:id="Rdffba31292d749e0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="WBS" sheetId="2" r:id="Re6fd5a7371714a92"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase 1 Gantt" sheetId="3" r:id="Rd054c57f8f6f4ad6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase 2 Gantt" sheetId="4" r:id="R1f7d7a418c1547e2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Milestones &amp; Decisions" sheetId="5" r:id="Rce610b1fe8764f00"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risks &amp; Assumptions" sheetId="6" r:id="R5e8884089e5b4af6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources &amp; Change Log" sheetId="7" r:id="R1b9173a071d049fa"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Team Calendar" sheetId="8" r:id="R6c225aa2e2c64a33"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fast Track Plan" sheetId="9" r:id="Re5931c8d10264a24"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Strategy" sheetId="10" r:id="R7fcf4a9d230b4577"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1762,7 +1762,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rb4f270c219a54f50"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R1138253bc980411d"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1792,7 +1792,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R0afa5321836a4e25"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R195beb5aca77490f"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -2495,7 +2495,7 @@
     <x:mergeCell ref="A18:V18"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd5409e5d48684c00"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R558bd9a4f7f840ff"/>
 </x:worksheet>
 </file>
 
@@ -4610,7 +4610,7 @@
       </x:c>
       <x:c r="Q29" s="195" t="str">
         <x:v>2026-09-23 Lead 결정으로 09-22에서 10-06(화)으로 조정. 같은 날 #30 보완·Sign-off와 #32 Close로 이어진다. G3 통과와 참석자 확정이 필요하다. 실제 상태·완료 판정은 유지한다.
-GitHub open/- · 10/19 사용자 비동기 증적 Review 방식/최종결과 한정 채택. 실제 기록 https://github.com/321Team/fds-project-baseline/issues/31#issuecomment-6265340124 · 실제 closed(completed) 2026-10-19T19:45:18+09:00. #30 Signoff/#32 Close 별도.</x:v>
+GitHub closed/completed · 10/19 사용자 비동기 증적 Review 방식/최종결과 한정 채택. 실제 기록 https://github.com/321Team/fds-project-baseline/issues/31#issuecomment-6265340124 · 실제 closed(completed) 2026-10-19T19:45:18+09:00. #30 Signoff/#32 Close 별도.</x:v>
       </x:c>
       <x:c r="R29" s="13" t="str">
         <x:v>https://github.com/321Team/fds-project-baseline/issues/31 · 실제종결 2026-10-19T19:45:18+09:00 · body SHA 74b462cf3f0a · 실제Review채택 https://github.com/321Team/fds-project-baseline/issues/31#issuecomment-6265340124</x:v>
@@ -7914,7 +7914,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbba67dac05554f84"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4c553cd8f0d945b3"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -25627,7 +25627,7 @@
       <x:c r="I10" s="195" t="str">
         <x:f>WBS!Q29</x:f>
         <x:v>2026-09-23 Lead 결정으로 09-22에서 10-06(화)으로 조정. 같은 날 #30 보완·Sign-off와 #32 Close로 이어진다. G3 통과와 참석자 확정이 필요하다. 실제 상태·완료 판정은 유지한다.
-GitHub open/- · 10/19 사용자 비동기 증적 Review 방식/최종결과 한정 채택. 실제 기록 https://github.com/321Team/fds-project-baseline/issues/31#issuecomment-6265340124 · 실제 closed(completed) 2026-10-19T19:45:18+09:00. #30 Signoff/#32 Close 별도.</x:v>
+GitHub closed/completed · 10/19 사용자 비동기 증적 Review 방식/최종결과 한정 채택. 실제 기록 https://github.com/321Team/fds-project-baseline/issues/31#issuecomment-6265340124 · 실제 closed(completed) 2026-10-19T19:45:18+09:00. #30 Signoff/#32 Close 별도.</x:v>
       </x:c>
       <x:c r="J10" s="195" t="str">
         <x:v>Lifecycle only; Runtime separate</x:v>

</xml_diff>

<commit_message>
docs: track Phase1 final Signoff and sequential Close (signed)
</commit_message>
<xml_diff>
--- a/audit/canonical-candidate-20261019/proposed/FDS_P1_WBS_Status_Candidate_20261019.xlsx
+++ b/audit/canonical-candidate-20261019/proposed/FDS_P1_WBS_Status_Candidate_20261019.xlsx
@@ -2,16 +2,16 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Executive Summary" sheetId="1" r:id="Rdffba31292d749e0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="WBS" sheetId="2" r:id="Re6fd5a7371714a92"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase 1 Gantt" sheetId="3" r:id="Rd054c57f8f6f4ad6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase 2 Gantt" sheetId="4" r:id="R1f7d7a418c1547e2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Milestones &amp; Decisions" sheetId="5" r:id="Rce610b1fe8764f00"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risks &amp; Assumptions" sheetId="6" r:id="R5e8884089e5b4af6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources &amp; Change Log" sheetId="7" r:id="R1b9173a071d049fa"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Team Calendar" sheetId="8" r:id="R6c225aa2e2c64a33"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fast Track Plan" sheetId="9" r:id="Re5931c8d10264a24"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Strategy" sheetId="10" r:id="R7fcf4a9d230b4577"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Executive Summary" sheetId="1" r:id="Ref76a872aaf04ca4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="WBS" sheetId="2" r:id="R4a9d341850de4a64"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase 1 Gantt" sheetId="3" r:id="R2083984d34a44232"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase 2 Gantt" sheetId="4" r:id="Rb38f25b7edc340b4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Milestones &amp; Decisions" sheetId="5" r:id="Re4133e09d12844d3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risks &amp; Assumptions" sheetId="6" r:id="R61cb0b33e0fe4ce4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources &amp; Change Log" sheetId="7" r:id="Rb5a58cd9f19840e9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Team Calendar" sheetId="8" r:id="Rf444d4bb0e7c4b8c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fast Track Plan" sheetId="9" r:id="R6856a1a934484d14"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Strategy" sheetId="10" r:id="R8d0fccce982f4c35"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1762,7 +1762,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R1138253bc980411d"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R0bfe7a70acaf4f6f"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1792,7 +1792,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R195beb5aca77490f"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R12a480a1265e41d5"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -2114,7 +2114,7 @@
         <x:v>P1 Close</x:v>
       </x:c>
       <x:c r="E4" s="199" t="str">
-        <x:v>Review 채택 완료 · Signoff 잔여</x:v>
+        <x:v>최종 Signoff 채택 · Close 대기</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="32" customHeight="1">
@@ -2372,7 +2372,7 @@
         <x:v>P1 Close</x:v>
       </x:c>
       <x:c r="C21" s="13" t="str">
-        <x:v>모듈·G1~G3·#31 조건부 Review 인수 완료. #30 Signoff/#32 Close 잔여.</x:v>
+        <x:v>#30 조건부 최종Signoff 실제 저장. 관리정합 후 #32 순차Close 승인, 아직 미실행.</x:v>
       </x:c>
       <x:c r="D21" s="195" t="str">
         <x:v>각 P1 Lead</x:v>
@@ -2495,7 +2495,7 @@
     <x:mergeCell ref="A18:V18"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R558bd9a4f7f840ff"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Raa9ce6b0c465405b"/>
 </x:worksheet>
 </file>
 
@@ -4546,11 +4546,10 @@
       </x:c>
       <x:c r="Q28" s="195" t="str">
         <x:v>10-06 하루에 Phase 1 Review/Close를 수행한다. 10-02 cutoff 이후 신규 Scope 확장은 하지 않고, 미완료 항목을 MET / NOT MET-RISK ACCEPTED / KNOWN ISSUE / APPROVED DEFERRED로 분류해 Owner·Due·Evidence를 고정한 뒤 #32 Close로 인계한다.
-10/6 Close 결과 미수신; 미충족/위험/Owner 인계.
-GitHub open/-</x:v>
+조건부 최종Signoff 2026-10-19T20:05:51.513852+09:00 · https://github.com/321Team/fds-project-baseline/issues/30#issuecomment-6265747689 · 기존RA/KI·이월 보존. GitHub open, 종결 전 추적 반영.</x:v>
       </x:c>
       <x:c r="R28" s="13" t="str">
-        <x:v>https://github.com/321Team/fds-project-baseline/issues/30 · 조회 2026-10-19T19:25 KST · body SHA adae54557399</x:v>
+        <x:v>https://github.com/321Team/fds-project-baseline/issues/30 · 실제 최종Signoff https://github.com/321Team/fds-project-baseline/issues/30#issuecomment-6265747689 · 판단 입력 b085e027</x:v>
       </x:c>
       <x:c r="S28" s="13" t="str">
         <x:f>IF(G28="Done","Done",IF(I28="","End TBD",IF(I28&lt;'Executive Summary'!$B$4,"Target elapsed",IF(H28&gt;'Executive Summary'!$B$4,"Upcoming","Active window"))))</x:f>
@@ -4673,7 +4672,7 @@
       </x:c>
       <x:c r="Q30" s="195" t="str">
         <x:v>2026-09-23 Lead 결정으로 10-06에 종결한다(Phase 1 진행 항목 #74·#75 등 10-06 계획 감안). #31 Review → #30 보완·Sign-off → Close 순으로 같은 날 진행하며, Close 판정 후 Phase 2 Start(#33)로 이어진다.
-GitHub open/-</x:v>
+A·B 실제 채택. #30 실제 서명 저장·후속 관리 정합 확인 후 순차 Close 승인, 현재 종결 대기. https://github.com/321Team/fds-project-baseline/issues/30#issuecomment-6265747689 · GitHub open.</x:v>
       </x:c>
       <x:c r="R30" s="13" t="str">
         <x:v>https://github.com/321Team/fds-project-baseline/issues/32 · 조회 2026-10-19T19:25 KST · body SHA be9aebeff65a</x:v>
@@ -7914,7 +7913,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4c553cd8f0d945b3"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3c65e093f9b14e56"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -25668,7 +25667,7 @@
       <x:c r="I11" s="195" t="str">
         <x:f>WBS!Q30</x:f>
         <x:v>2026-09-23 Lead 결정으로 10-06에 종결한다(Phase 1 진행 항목 #74·#75 등 10-06 계획 감안). #31 Review → #30 보완·Sign-off → Close 순으로 같은 날 진행하며, Close 판정 후 Phase 2 Start(#33)로 이어진다.
-GitHub open/-</x:v>
+A·B 실제 채택. #30 실제 서명 저장·후속 관리 정합 확인 후 순차 Close 승인, 현재 종결 대기. https://github.com/321Team/fds-project-baseline/issues/30#issuecomment-6265747689 · GitHub open.</x:v>
       </x:c>
       <x:c r="J11" s="195" t="str">
         <x:v>Lifecycle only; Runtime separate</x:v>

</xml_diff>

<commit_message>
docs: track Phase1 final Signoff and sequential Close (closed30)
</commit_message>
<xml_diff>
--- a/audit/canonical-candidate-20261019/proposed/FDS_P1_WBS_Status_Candidate_20261019.xlsx
+++ b/audit/canonical-candidate-20261019/proposed/FDS_P1_WBS_Status_Candidate_20261019.xlsx
@@ -2,16 +2,16 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Executive Summary" sheetId="1" r:id="Ref76a872aaf04ca4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="WBS" sheetId="2" r:id="R4a9d341850de4a64"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase 1 Gantt" sheetId="3" r:id="R2083984d34a44232"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase 2 Gantt" sheetId="4" r:id="Rb38f25b7edc340b4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Milestones &amp; Decisions" sheetId="5" r:id="Re4133e09d12844d3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risks &amp; Assumptions" sheetId="6" r:id="R61cb0b33e0fe4ce4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources &amp; Change Log" sheetId="7" r:id="Rb5a58cd9f19840e9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Team Calendar" sheetId="8" r:id="Rf444d4bb0e7c4b8c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fast Track Plan" sheetId="9" r:id="R6856a1a934484d14"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Strategy" sheetId="10" r:id="R8d0fccce982f4c35"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Executive Summary" sheetId="1" r:id="Rb94e5da2c98e4306"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="WBS" sheetId="2" r:id="Rf8f07948ccac4c1f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase 1 Gantt" sheetId="3" r:id="Rc6ced55e7a204252"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase 2 Gantt" sheetId="4" r:id="Ra60f709b2c8f4423"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Milestones &amp; Decisions" sheetId="5" r:id="Rdabf5121e8c34e3b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risks &amp; Assumptions" sheetId="6" r:id="R171d5251771e4226"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources &amp; Change Log" sheetId="7" r:id="Rba66a60c22bc4219"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Team Calendar" sheetId="8" r:id="R821f4863ecbf460f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fast Track Plan" sheetId="9" r:id="Re0f6890d6e684800"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Strategy" sheetId="10" r:id="Rc7d64b73ef1248ff"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1762,7 +1762,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R0bfe7a70acaf4f6f"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R4a8d150284674d49"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1792,7 +1792,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R12a480a1265e41d5"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rbc4d6ce0c2e044c4"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -2114,7 +2114,7 @@
         <x:v>P1 Close</x:v>
       </x:c>
       <x:c r="E4" s="199" t="str">
-        <x:v>최종 Signoff 채택 · Close 대기</x:v>
+        <x:v>Signoff 종결 · 전체 Close 대기</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="32" customHeight="1">
@@ -2228,7 +2228,7 @@
       </x:c>
       <x:c r="B12" s="13" t="n">
         <x:f>COUNTIF(WBS!$G$4:$G$81,A12)</x:f>
-        <x:v>43</x:v>
+        <x:v>44</x:v>
       </x:c>
       <x:c r="D12" s="13" t="inlineStr">
         <x:is>
@@ -2248,7 +2248,7 @@
       </x:c>
       <x:c r="B13" s="13" t="n">
         <x:f>COUNTIF(WBS!$G$4:$G$81,A13)</x:f>
-        <x:v>12</x:v>
+        <x:v>11</x:v>
       </x:c>
       <x:c r="D13" s="13" t="inlineStr">
         <x:is>
@@ -2372,7 +2372,7 @@
         <x:v>P1 Close</x:v>
       </x:c>
       <x:c r="C21" s="13" t="str">
-        <x:v>#30 조건부 최종Signoff 실제 저장. 관리정합 후 #32 순차Close 승인, 아직 미실행.</x:v>
+        <x:v>#30 조건부 최종Signoff 종결·추적 반영. #32 원조건 확인 후 순차 Close 진행.</x:v>
       </x:c>
       <x:c r="D21" s="195" t="str">
         <x:v>각 P1 Lead</x:v>
@@ -2495,7 +2495,7 @@
     <x:mergeCell ref="A18:V18"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Raa9ce6b0c465405b"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R96b4acf6f6fc4d6b"/>
 </x:worksheet>
 </file>
 
@@ -4513,7 +4513,7 @@
         <x:v>P0</x:v>
       </x:c>
       <x:c r="G28" s="13" t="str">
-        <x:v>In Progress</x:v>
+        <x:v>Done</x:v>
       </x:c>
       <x:c r="H28" s="191" t="n">
         <x:v>46301</x:v>
@@ -4546,14 +4546,14 @@
       </x:c>
       <x:c r="Q28" s="195" t="str">
         <x:v>10-06 하루에 Phase 1 Review/Close를 수행한다. 10-02 cutoff 이후 신규 Scope 확장은 하지 않고, 미완료 항목을 MET / NOT MET-RISK ACCEPTED / KNOWN ISSUE / APPROVED DEFERRED로 분류해 Owner·Due·Evidence를 고정한 뒤 #32 Close로 인계한다.
-조건부 최종Signoff 2026-10-19T20:05:51.513852+09:00 · https://github.com/321Team/fds-project-baseline/issues/30#issuecomment-6265747689 · 기존RA/KI·이월 보존. GitHub open, 종결 전 추적 반영.</x:v>
+조건부 최종 Signoff 채택·실제 closed(completed) 2026-10-19T20:10:15+09:00 · https://github.com/321Team/fds-project-baseline/issues/30#issuecomment-6265747689 · 기존 기술 미검증·Owner/재검토·계획 보존.</x:v>
       </x:c>
       <x:c r="R28" s="13" t="str">
-        <x:v>https://github.com/321Team/fds-project-baseline/issues/30 · 실제 최종Signoff https://github.com/321Team/fds-project-baseline/issues/30#issuecomment-6265747689 · 판단 입력 b085e027</x:v>
+        <x:v>https://github.com/321Team/fds-project-baseline/issues/30 · 실제종결 2026-10-19T20:10:15+09:00 · body SHA 5302bed40005 · 실제판정 https://github.com/321Team/fds-project-baseline/issues/30#issuecomment-6265747689</x:v>
       </x:c>
       <x:c r="S28" s="13" t="str">
         <x:f>IF(G28="Done","Done",IF(I28="","End TBD",IF(I28&lt;'Executive Summary'!$B$4,"Target elapsed",IF(H28&gt;'Executive Summary'!$B$4,"Upcoming","Active window"))))</x:f>
-        <x:v>Target elapsed</x:v>
+        <x:v>Done</x:v>
       </x:c>
     </x:row>
     <x:row r="29" ht="110" customHeight="1">
@@ -7913,7 +7913,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3c65e093f9b14e56"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc5bdf2d26e8b4c43"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -11879,7 +11879,7 @@
       </x:c>
       <x:c r="C27" s="195" t="str">
         <x:f>WBS!G28</x:f>
-        <x:v>In Progress</x:v>
+        <x:v>Done</x:v>
       </x:c>
       <x:c r="D27" s="225" t="n">
         <x:f>WBS!H28</x:f>

</xml_diff>

<commit_message>
docs: track Phase1 final Signoff and sequential Close (closed32)
</commit_message>
<xml_diff>
--- a/audit/canonical-candidate-20261019/proposed/FDS_P1_WBS_Status_Candidate_20261019.xlsx
+++ b/audit/canonical-candidate-20261019/proposed/FDS_P1_WBS_Status_Candidate_20261019.xlsx
@@ -2,16 +2,16 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Executive Summary" sheetId="1" r:id="Rb94e5da2c98e4306"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="WBS" sheetId="2" r:id="Rf8f07948ccac4c1f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase 1 Gantt" sheetId="3" r:id="Rc6ced55e7a204252"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase 2 Gantt" sheetId="4" r:id="Ra60f709b2c8f4423"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Milestones &amp; Decisions" sheetId="5" r:id="Rdabf5121e8c34e3b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risks &amp; Assumptions" sheetId="6" r:id="R171d5251771e4226"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources &amp; Change Log" sheetId="7" r:id="Rba66a60c22bc4219"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Team Calendar" sheetId="8" r:id="R821f4863ecbf460f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fast Track Plan" sheetId="9" r:id="Re0f6890d6e684800"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Strategy" sheetId="10" r:id="Rc7d64b73ef1248ff"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Executive Summary" sheetId="1" r:id="R28958dcf4e774341"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="WBS" sheetId="2" r:id="Rf0d8d5be11174590"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase 1 Gantt" sheetId="3" r:id="R0eb3bb0b363644a0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase 2 Gantt" sheetId="4" r:id="Rf1feeb5647df4c0a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Milestones &amp; Decisions" sheetId="5" r:id="Rd65f4587df744d62"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risks &amp; Assumptions" sheetId="6" r:id="R54fbce9028a94d7c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources &amp; Change Log" sheetId="7" r:id="R7d88122512e1443f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Team Calendar" sheetId="8" r:id="R0db30c13745f433b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fast Track Plan" sheetId="9" r:id="Raa877322206244d9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Strategy" sheetId="10" r:id="Rbad9ad8b00664a07"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1762,7 +1762,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R4a8d150284674d49"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R6a37b366950c498e"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1792,7 +1792,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rbc4d6ce0c2e044c4"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R620212eb909544e9"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -2114,7 +2114,7 @@
         <x:v>P1 Close</x:v>
       </x:c>
       <x:c r="E4" s="199" t="str">
-        <x:v>Signoff 종결 · 전체 Close 대기</x:v>
+        <x:v>Phase1 조건부 Close 완료</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="32" customHeight="1">
@@ -2228,7 +2228,7 @@
       </x:c>
       <x:c r="B12" s="13" t="n">
         <x:f>COUNTIF(WBS!$G$4:$G$81,A12)</x:f>
-        <x:v>44</x:v>
+        <x:v>45</x:v>
       </x:c>
       <x:c r="D12" s="13" t="inlineStr">
         <x:is>
@@ -2288,7 +2288,7 @@
       </x:c>
       <x:c r="B15" s="13" t="n">
         <x:f>COUNTIF(WBS!$G$4:$G$81,A15)</x:f>
-        <x:v>20</x:v>
+        <x:v>19</x:v>
       </x:c>
     </x:row>
     <x:row r="16">
@@ -2372,7 +2372,7 @@
         <x:v>P1 Close</x:v>
       </x:c>
       <x:c r="C21" s="13" t="str">
-        <x:v>#30 조건부 최종Signoff 종결·추적 반영. #32 원조건 확인 후 순차 Close 진행.</x:v>
+        <x:v>Phase1 #30 Signoff·#32 전체Close 종결. 기존RA/KI/승인이월·재검토 유지. 새 정본 발행은 별도.</x:v>
       </x:c>
       <x:c r="D21" s="195" t="str">
         <x:v>각 P1 Lead</x:v>
@@ -2495,7 +2495,7 @@
     <x:mergeCell ref="A18:V18"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R96b4acf6f6fc4d6b"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5010cd8f35cd4ebd"/>
 </x:worksheet>
 </file>
 
@@ -4549,7 +4549,7 @@
 조건부 최종 Signoff 채택·실제 closed(completed) 2026-10-19T20:10:15+09:00 · https://github.com/321Team/fds-project-baseline/issues/30#issuecomment-6265747689 · 기존 기술 미검증·Owner/재검토·계획 보존.</x:v>
       </x:c>
       <x:c r="R28" s="13" t="str">
-        <x:v>https://github.com/321Team/fds-project-baseline/issues/30 · 실제종결 2026-10-19T20:10:15+09:00 · body SHA 5302bed40005 · 실제판정 https://github.com/321Team/fds-project-baseline/issues/30#issuecomment-6265747689</x:v>
+        <x:v>https://github.com/321Team/fds-project-baseline/issues/30 · 실제종결 2026-10-19T20:10:15+09:00 · body SHA 352142fde228 · 실제판정 https://github.com/321Team/fds-project-baseline/issues/30#issuecomment-6265747689</x:v>
       </x:c>
       <x:c r="S28" s="13" t="str">
         <x:f>IF(G28="Done","Done",IF(I28="","End TBD",IF(I28&lt;'Executive Summary'!$B$4,"Target elapsed",IF(H28&gt;'Executive Summary'!$B$4,"Upcoming","Active window"))))</x:f>
@@ -4639,7 +4639,7 @@
         <x:v>P0</x:v>
       </x:c>
       <x:c r="G30" s="13" t="str">
-        <x:v>To Do</x:v>
+        <x:v>Done</x:v>
       </x:c>
       <x:c r="H30" s="191" t="n">
         <x:v>46301</x:v>
@@ -4672,14 +4672,14 @@
       </x:c>
       <x:c r="Q30" s="195" t="str">
         <x:v>2026-09-23 Lead 결정으로 10-06에 종결한다(Phase 1 진행 항목 #74·#75 등 10-06 계획 감안). #31 Review → #30 보완·Sign-off → Close 순으로 같은 날 진행하며, Close 판정 후 Phase 2 Start(#33)로 이어진다.
-A·B 실제 채택. #30 실제 서명 저장·후속 관리 정합 확인 후 순차 Close 승인, 현재 종결 대기. https://github.com/321Team/fds-project-baseline/issues/30#issuecomment-6265747689 · GitHub open.</x:v>
+기존 RA/KI·이월 보존한 Phase1 전체 Close 채택·실제 closed(completed) 2026-10-19T20:12:53+09:00 · https://github.com/321Team/fds-project-baseline/issues/32#issuecomment-6265873856 · 기존 기술 미검증·Owner/재검토·계획 보존.</x:v>
       </x:c>
       <x:c r="R30" s="13" t="str">
-        <x:v>https://github.com/321Team/fds-project-baseline/issues/32 · 조회 2026-10-19T19:25 KST · body SHA be9aebeff65a</x:v>
+        <x:v>https://github.com/321Team/fds-project-baseline/issues/32 · 실제종결 2026-10-19T20:12:53+09:00 · body SHA 1101f33ab227 · 실제판정 https://github.com/321Team/fds-project-baseline/issues/32#issuecomment-6265873856</x:v>
       </x:c>
       <x:c r="S30" s="13" t="str">
         <x:f>IF(G30="Done","Done",IF(I30="","End TBD",IF(I30&lt;'Executive Summary'!$B$4,"Target elapsed",IF(H30&gt;'Executive Summary'!$B$4,"Upcoming","Active window"))))</x:f>
-        <x:v>Target elapsed</x:v>
+        <x:v>Done</x:v>
       </x:c>
     </x:row>
     <x:row r="31" ht="110" customHeight="1">
@@ -7913,7 +7913,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc5bdf2d26e8b4c43"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8bf03b2819094d6d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -12201,7 +12201,7 @@
       </x:c>
       <x:c r="C29" s="195" t="str">
         <x:f>WBS!G30</x:f>
-        <x:v>To Do</x:v>
+        <x:v>Done</x:v>
       </x:c>
       <x:c r="D29" s="225" t="n">
         <x:f>WBS!H30</x:f>
@@ -25647,7 +25647,7 @@
       </x:c>
       <x:c r="D11" s="13" t="str">
         <x:f>WBS!G30</x:f>
-        <x:v>To Do</x:v>
+        <x:v>Done</x:v>
       </x:c>
       <x:c r="E11" s="191" t="n">
         <x:f>WBS!H30</x:f>
@@ -25667,7 +25667,7 @@
       <x:c r="I11" s="195" t="str">
         <x:f>WBS!Q30</x:f>
         <x:v>2026-09-23 Lead 결정으로 10-06에 종결한다(Phase 1 진행 항목 #74·#75 등 10-06 계획 감안). #31 Review → #30 보완·Sign-off → Close 순으로 같은 날 진행하며, Close 판정 후 Phase 2 Start(#33)로 이어진다.
-A·B 실제 채택. #30 실제 서명 저장·후속 관리 정합 확인 후 순차 Close 승인, 현재 종결 대기. https://github.com/321Team/fds-project-baseline/issues/30#issuecomment-6265747689 · GitHub open.</x:v>
+기존 RA/KI·이월 보존한 Phase1 전체 Close 채택·실제 closed(completed) 2026-10-19T20:12:53+09:00 · https://github.com/321Team/fds-project-baseline/issues/32#issuecomment-6265873856 · 기존 기술 미검증·Owner/재검토·계획 보존.</x:v>
       </x:c>
       <x:c r="J11" s="195" t="str">
         <x:v>Lifecycle only; Runtime separate</x:v>

</xml_diff>